<commit_message>
feat: add AI audio podcast generation and Telegram voice delivery
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -565,10 +565,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>241237</v>
+        <v>241243</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>49444</v>
+        <v>49447</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -608,10 +608,10 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>154427</v>
+        <v>154429</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24410</v>
+        <v>24411</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -654,7 +654,7 @@
         <v>154239</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10016</v>
+        <v>10017</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>150004</v>
+        <v>150006</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>24166</v>
@@ -733,10 +733,10 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143341</v>
+        <v>143342</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34825</v>
+        <v>34826</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -779,7 +779,7 @@
         <v>136014</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>20002</v>
+        <v>20003</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>48781</v>
+        <v>48782</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>4830</v>
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13614</v>
+        <v>13615</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1618</v>
@@ -1069,10 +1069,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>247875</v>
+        <v>247890</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>37349</v>
+        <v>37351</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>124546</v>
+        <v>124573</v>
       </c>
       <c r="E16" s="5" t="n">
         <v>6719</v>
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>114630</v>
+        <v>114633</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>11138</v>
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>210065</v>
+        <v>210071</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>21353</v>
@@ -1366,7 +1366,7 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187114</v>
+        <v>187113</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>46039</v>
@@ -1412,7 +1412,7 @@
         <v>180124</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17682</v>
+        <v>17683</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>176356</v>
+        <v>176359</v>
       </c>
       <c r="E24" s="5" t="n">
         <v>9650</v>

</xml_diff>

<commit_message>
feat(ultimate): complete 5 major skills (AI Insight, Velocity, Interactive Bot, Podcast, GitHub Pages)
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -568,7 +568,7 @@
         <v>241243</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>49447</v>
+        <v>49448</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>150006</v>
+        <v>150008</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>24166</v>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5702</v>
+        <v>5701</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>714</v>
@@ -1069,10 +1069,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>247890</v>
+        <v>247893</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>37351</v>
+        <v>37352</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>124573</v>
+        <v>124583</v>
       </c>
       <c r="E16" s="5" t="n">
         <v>6719</v>
@@ -1155,10 +1155,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>114633</v>
+        <v>114635</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11138</v>
+        <v>11139</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>176359</v>
+        <v>176364</v>
       </c>
       <c r="E24" s="5" t="n">
         <v>9650</v>

</xml_diff>

<commit_message>
refactor: translate all reports, UI, podcast, and bot to English
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -480,14 +480,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -565,14 +567,14 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>241243</v>
+        <v>241245</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>49448</v>
+        <v>49449</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -582,12 +584,12 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>ai, ai-agent, ai-agents, anthropic, chatgpt</t>
+          <t>The agent that grows with you</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/NousResearch/hermes-agent</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>
@@ -611,11 +613,11 @@
         <v>154429</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24411</v>
+        <v>24410</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -625,12 +627,12 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>agent, agentic-ai, agentic-framework, agentic-workflow, ai</t>
+          <t>Build Agentic workflows, RAG pipelines, with rich AI model and tool support on one collaborative workspace. Deploy on cloud, VPC, or self-hosted, so teams move from prototype to production without rebuilding the stack.</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/langgenius/dify</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>
@@ -658,7 +660,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -668,12 +670,12 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>agents, chatgpt, generative-ai, large-language-models, multiagent</t>
+          <t>Langflow is a powerful tool for building and deploying AI-powered agents and workflows.</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/langflow-ai/langflow</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>
@@ -701,7 +703,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Shell</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -709,10 +711,14 @@
           <t>A complete AI agency at your fingertips - From frontend wizards to Reddit community ninjas, from whimsy injectors to reality checkers. Each agent is a specialized expert with personality, processes, and proven deliverables.</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>A complete AI agency at your fingertips - From frontend wizards to Reddit community ninjas, from whimsy injectors to reality checkers. Each agent is a specialized expert with personality, processes, and proven deliverables.</t>
+        </is>
+      </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/msitarzewski/agency-agents</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>
@@ -740,7 +746,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -750,12 +756,12 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>ai, bolt, cluely, copilot, cursor</t>
+          <t>FULL Augment Code, Claude Code, Cluely, CodeBuddy, Comet, Cursor, Devin AI, Junie, Kiro, Leap.new, Lovable, Manus, NotionAI, Orchids.app, Perplexity, Poke, Qoder, Replit, Same.dev, Trae, Traycer AI, VSCode Agent, Warp.dev, Windsurf, Xcode, Z.ai Code, Dia &amp; v0. (And other Open Sourced) System Prompts, Internal Tools &amp; AI Models</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/x1xhlol/system-prompts-and-models-of-ai-tools</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>
@@ -783,7 +789,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -793,12 +799,12 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>agents, llms, python, rag</t>
+          <t>100+ AI Agents, Agent Skills and RAG Apps - Free and Open Source.</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/Shubhamsaboo/awesome-llm-apps</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>
@@ -826,7 +832,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -836,12 +842,12 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>ai-companion, ai-vtuber, airi, digital-life, grok-companion</t>
+          <t>💖🧸 Self hosted, you-owned Grok Companion, a container of souls of waifu, cyber livings to bring them into our worlds, wishing to achieve Neuro-sama's altitude. Capable of realtime voice chat, Minecraft, Factorio playing. Web / macOS / Windows supported.</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/moeru-ai/airi</t>
+          <t>Create Virtual Companions, VTubers &amp; Voice-Driven Characters</t>
         </is>
       </c>
     </row>
@@ -869,7 +875,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -879,12 +885,12 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>ai, ai-companion, ai-vtuber, ai-waifu, chatbots</t>
+          <t>Talk to any LLM with hands-free voice interaction, voice interruption, and Live2D taking face running locally across platforms</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/Open-LLM-VTuber/Open-LLM-VTuber</t>
+          <t>Create Virtual Companions, VTubers &amp; Voice-Driven Characters</t>
         </is>
       </c>
     </row>
@@ -912,7 +918,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -922,12 +928,12 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>javascript-plugin, live2d</t>
+          <t>把萌萌哒的看板娘抱回家 (ノ≧∇≦)ノ | Live2D widget for web platform</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/stevenjoezhang/live2d-widget</t>
+          <t>Create Virtual Companions, VTubers &amp; Voice-Driven Characters</t>
         </is>
       </c>
     </row>
@@ -955,7 +961,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>CSS</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -963,10 +969,14 @@
           <t xml:space="preserve">High-quality PNGs for logos I made for fun </t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High-quality PNGs for logos I made for fun </t>
+        </is>
+      </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/Aikoyori/ProgrammingVTuberLogos</t>
+          <t>Create Virtual Companions, VTubers &amp; Voice-Driven Characters</t>
         </is>
       </c>
     </row>
@@ -994,7 +1004,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1004,12 +1014,12 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>face-detection, hand-detection, mediapipe-facemesh, mediapipe-hands, mediapipe-pose</t>
+          <t>Blendshape and kinematics calculator for Mediapipe/Tensorflow.js Face, Eyes, Pose, and Finger tracking models.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/yeemachine/kalidokit</t>
+          <t>Create Virtual Companions, VTubers &amp; Voice-Driven Characters</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1047,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>JavaScript</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1045,10 +1055,14 @@
           <t>Add the Sseexxyyy live2d to your hexo!</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Add the Sseexxyyy live2d to your hexo!</t>
+        </is>
+      </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/EYHN/hexo-helper-live2d</t>
+          <t>Create Virtual Companions, VTubers &amp; Voice-Driven Characters</t>
         </is>
       </c>
     </row>
@@ -1069,14 +1083,14 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>247893</v>
+        <v>247896</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>37352</v>
+        <v>37354</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>JavaScript</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1086,12 +1100,12 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>ai-agents, anthropic, claude, claude-code, developer-tools</t>
+          <t>The agent harness performance optimization system. Skills, instincts, memory, security, and research-first development for Claude Code, Codex, Opencode, Cursor and beyond.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/affaan-m/ECC</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>
@@ -1112,14 +1126,14 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>124583</v>
+        <v>124590</v>
       </c>
       <c r="E16" s="5" t="n">
         <v>6719</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>JavaScript</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1129,12 +1143,12 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>agent-skills, ai-agents, claude, claude-code, claude-code-plugin</t>
+          <t>Makes your AI agent think like the laziest senior dev in the room. The best code is the code you never wrote.</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/DietrichGebert/ponytail</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1176,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1172,12 +1186,12 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>ai-agents, antigravity, ast, claude-code, code-analysis</t>
+          <t>Turn any codebase, with its docs, SQL schemas, configs, and PDFs, into a queryable knowledge graph. A /graphify skill for Claude Code, Cursor, Codex, and Gemini CLI: local deterministic AST parsing, every edge explained, no vector store.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/Graphify-Labs/graphify</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1219,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1215,12 +1229,12 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>automation, chrome, chromium, developer-tools, firefox</t>
+          <t>JavaScript API for Chrome and Firefox</t>
         </is>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/puppeteer/puppeteer</t>
+          <t>Developer Productivity, AST Code Intelligence &amp; Terminal Tools</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1262,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1258,12 +1272,12 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>agent, artificial-intelligence, chatgpt, claude-ai, cli</t>
+          <t>🙌 OpenHands: AI-Driven Development</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/OpenHands/OpenHands</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>
@@ -1291,7 +1305,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1301,12 +1315,12 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>api, api-client, api-rest, api-testing, developer-tools</t>
+          <t>Open-Source API Development Ecosystem • https://hoppscotch.io • Offline, On-Prem &amp; Cloud • Web, Desktop &amp; CLI • Open-Source Alternative to Postman, Insomnia</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/hoppscotch/hoppscotch</t>
+          <t>Developer Productivity, AST Code Intelligence &amp; Terminal Tools</t>
         </is>
       </c>
     </row>
@@ -1327,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>210071</v>
+        <v>210072</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>21353</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1342,10 +1356,14 @@
           <t>A single CLAUDE.md file to improve Claude Code behavior, derived from Andrej Karpathy's observations on LLM coding pitfalls.</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>A single CLAUDE.md file to improve Claude Code behavior, derived from Andrej Karpathy's observations on LLM coding pitfalls.</t>
+        </is>
+      </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/multica-ai/andrej-karpathy-skills</t>
+          <t>Deploy Large Language Models, RAG Pipelines &amp; Audio Vision Systems</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1391,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1383,12 +1401,12 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>agentic-ai, agents, ai, artificial-intelligence, autonomous-agents</t>
+          <t>AutoGPT is the vision of accessible AI for everyone, to use and to build on. Our mission is to provide the tools, so that you can focus on what matters.</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/Significant-Gravitas/AutoGPT</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1434,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Go</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1426,12 +1444,12 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>deepseek, gemma, gemma3, glm, go</t>
+          <t>Get up and running with Kimi-K2.6, GLM-5.2, MiniMax, DeepSeek, gpt-oss, Qwen, Gemma and other models.</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/ollama/ollama</t>
+          <t>Deploy Large Language Models, RAG Pipelines &amp; Audio Vision Systems</t>
         </is>
       </c>
     </row>
@@ -1452,14 +1470,14 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>176364</v>
+        <v>176367</v>
       </c>
       <c r="E24" s="5" t="n">
         <v>9650</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1469,12 +1487,12 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>ai, ai-agents, ai-crawler, ai-scraping, ai-search</t>
+          <t>The context API to search, scrape, and interact with the web at scale. 🔥</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/firecrawl/firecrawl</t>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add interactive Visual Analytics charts and KPI metrics to Web Dashboard
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -570,7 +570,7 @@
         <v>241245</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>49449</v>
+        <v>49450</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>154429</v>
+        <v>154430</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>24410</v>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143342</v>
+        <v>143341</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>34826</v>
@@ -785,7 +785,7 @@
         <v>136014</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>20003</v>
+        <v>20002</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -828,7 +828,7 @@
         <v>48782</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4830</v>
+        <v>4831</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13615</v>
+        <v>13614</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1618</v>
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>247896</v>
+        <v>247899</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>37354</v>
+        <v>37355</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>124590</v>
+        <v>124593</v>
       </c>
       <c r="E16" s="5" t="n">
         <v>6719</v>
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>210072</v>
+        <v>210074</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>21353</v>
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>176367</v>
+        <v>176368</v>
       </c>
       <c r="E24" s="5" t="n">
         <v>9650</v>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-11]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GitHub Radar Archive" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="GitHub Radar Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>241245</v>
+        <v>244429</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>49450</v>
+        <v>50605</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>154430</v>
+        <v>155418</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24410</v>
+        <v>24548</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>154239</v>
+        <v>154576</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10017</v>
+        <v>10063</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>150008</v>
+        <v>151654</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24166</v>
+        <v>24425</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>🔥 Supernova (+1000⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143341</v>
+        <v>143533</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34826</v>
+        <v>34812</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+192⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -782,14 +782,14 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>136014</v>
+        <v>137142</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>20002</v>
+        <v>20162</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>🔥 Supernova (+1000⭐)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>48782</v>
+        <v>49040</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4831</v>
+        <v>4857</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+258⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13614</v>
+        <v>13704</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1618</v>
+        <v>1632</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+90⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>Talk to any LLM with hands-free voice interaction, voice interruption, and Live2D taking face running locally across platforms</t>
+          <t>Talk to any LLM with hands-free voice interaction, voice interruption, and Live2D avatar running locally across platforms</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10935</v>
+        <v>10948</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2605</v>
+        <v>2603</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+13⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6238</v>
+        <v>6237</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>301</v>
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5701</v>
+        <v>5703</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>247899</v>
+        <v>256213</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>37355</v>
+        <v>38343</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,14 +1126,14 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>124593</v>
+        <v>135412</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>6719</v>
+        <v>7260</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>🔥 Supernova (+1000⭐)</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>114635</v>
+        <v>116894</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11139</v>
+        <v>11318</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>🔥 Supernova (+1000⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95541</v>
+        <v>95574</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9577</v>
+        <v>9570</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+33⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>86155</v>
+        <v>87388</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11297</v>
+        <v>11457</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>🔥 Supernova (+1000⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1284,7 +1284,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1298,14 +1298,14 @@
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>80198</v>
+        <v>80283</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>6081</v>
+        <v>6099</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+85⭐)</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>210074</v>
+        <v>212238</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21353</v>
+        <v>21525</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>🔥 Supernova (+1000⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187113</v>
+        <v>187257</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46039</v>
+        <v>46022</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+144⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>180124</v>
+        <v>180656</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17683</v>
+        <v>17813</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,14 +1470,14 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>176368</v>
+        <v>179020</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9650</v>
+        <v>9741</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>🔥 Supernova (+1000⭐)</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-12]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>244429</v>
+        <v>244618</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>50605</v>
+        <v>50709</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>155418</v>
+        <v>155463</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24548</v>
+        <v>24554</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+45⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>154576</v>
+        <v>154603</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10063</v>
+        <v>10068</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+27⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>151654</v>
+        <v>151739</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24425</v>
+        <v>24433</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>🔥 Supernova (+1000⭐)</t>
+          <t>📈 Trending (+85⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143533</v>
+        <v>143547</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34812</v>
+        <v>34813</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+192⭐)</t>
+          <t>📈 Trending (+14⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -782,14 +782,14 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>137142</v>
+        <v>137249</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>20162</v>
+        <v>20195</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>🔥 Supernova (+1000⭐)</t>
+          <t>📈 Trending (+107⭐)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49040</v>
+        <v>49052</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4857</v>
+        <v>4860</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+258⭐)</t>
+          <t>📈 Trending (+12⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13704</v>
+        <v>13709</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1632</v>
+        <v>1635</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+90⭐)</t>
+          <t>📈 Trending (+5⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10948</v>
+        <v>10949</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2603</v>
+        <v>2602</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+13⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>256213</v>
+        <v>256545</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>38343</v>
+        <v>38392</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,14 +1126,14 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>135412</v>
+        <v>135857</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7260</v>
+        <v>7278</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>🔥 Supernova (+1000⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>116894</v>
+        <v>117031</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11318</v>
+        <v>11329</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>🔥 Supernova (+1000⭐)</t>
+          <t>📈 Trending (+137⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95574</v>
+        <v>95577</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9570</v>
+        <v>9571</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+33⭐)</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>87388</v>
+        <v>87555</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11457</v>
+        <v>11464</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>🔥 Supernova (+1000⭐)</t>
+          <t>📈 Trending (+167⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1284,7 +1284,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1298,14 +1298,14 @@
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>80283</v>
+        <v>80287</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>6099</v>
+        <v>6100</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+85⭐)</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>212238</v>
+        <v>212394</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21525</v>
+        <v>21539</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>🔥 Supernova (+1000⭐)</t>
+          <t>📈 Trending (+156⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187257</v>
+        <v>187270</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>46022</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+144⭐)</t>
+          <t>📈 Trending (+13⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>180656</v>
+        <v>180699</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17813</v>
+        <v>17817</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+43⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,14 +1470,14 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>179020</v>
+        <v>179235</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9741</v>
+        <v>9751</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>🔥 Supernova (+1000⭐)</t>
+          <t>📈 Trending (+215⭐)</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-13]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>244618</v>
+        <v>244909</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>50709</v>
+        <v>50831</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>155463</v>
+        <v>155554</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24554</v>
+        <v>24570</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+45⭐)</t>
+          <t>📈 Trending (+91⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>154603</v>
+        <v>154679</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10068</v>
+        <v>10082</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+27⭐)</t>
+          <t>📈 Trending (+76⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>151739</v>
+        <v>151942</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24433</v>
+        <v>24478</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+85⭐)</t>
+          <t>📈 Trending (+203⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143547</v>
+        <v>143572</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34813</v>
+        <v>34812</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+14⭐)</t>
+          <t>📈 Trending (+25⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -782,14 +782,14 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>137249</v>
+        <v>137643</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>20195</v>
+        <v>20235</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+107⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49052</v>
+        <v>49080</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4860</v>
+        <v>4865</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+12⭐)</t>
+          <t>📈 Trending (+28⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13709</v>
+        <v>13713</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1635</v>
+        <v>1638</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+5⭐)</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10949</v>
+        <v>10950</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2602</v>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>256545</v>
+        <v>257140</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>38392</v>
+        <v>38475</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>135857</v>
+        <v>136652</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7278</v>
+        <v>7328</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>117031</v>
+        <v>116257</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11329</v>
+        <v>11361</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+137⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95577</v>
+        <v>95579</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>9571</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>87555</v>
+        <v>87690</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11464</v>
+        <v>11489</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+167⭐)</t>
+          <t>📈 Trending (+135⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1284,7 +1284,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1298,14 +1298,14 @@
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>80287</v>
+        <v>80301</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>6100</v>
+        <v>6102</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+4⭐)</t>
+          <t>📈 Trending (+14⭐)</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>212394</v>
+        <v>212619</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21539</v>
+        <v>21552</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+156⭐)</t>
+          <t>📈 Trending (+225⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187270</v>
+        <v>187289</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46022</v>
+        <v>46019</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+13⭐)</t>
+          <t>📈 Trending (+19⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>180699</v>
+        <v>180761</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17817</v>
+        <v>17833</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+43⭐)</t>
+          <t>📈 Trending (+62⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,14 +1470,14 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>179235</v>
+        <v>179607</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9751</v>
+        <v>9766</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+215⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-14]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>244909</v>
+        <v>245183</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>50831</v>
+        <v>51004</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>155554</v>
+        <v>155628</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24570</v>
+        <v>24577</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+91⭐)</t>
+          <t>📈 Trending (+74⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>154679</v>
+        <v>154748</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10082</v>
+        <v>10083</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+76⭐)</t>
+          <t>📈 Trending (+69⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>151942</v>
+        <v>152151</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24478</v>
+        <v>24513</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+203⭐)</t>
+          <t>📈 Trending (+209⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143572</v>
+        <v>143603</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>34812</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+25⭐)</t>
+          <t>📈 Trending (+31⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -782,10 +782,10 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>137643</v>
+        <v>137973</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>20235</v>
+        <v>20276</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49080</v>
+        <v>49110</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4865</v>
+        <v>4867</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+28⭐)</t>
+          <t>📈 Trending (+30⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13713</v>
+        <v>13726</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1638</v>
+        <v>1640</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+4⭐)</t>
+          <t>📈 Trending (+13⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10950</v>
+        <v>10955</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2602</v>
+        <v>2603</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+5⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6237</v>
+        <v>6235</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>301</v>
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5703</v>
+        <v>5704</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>713</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>257140</v>
+        <v>257785</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>38475</v>
+        <v>38552</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>136652</v>
+        <v>137393</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7328</v>
+        <v>7381</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>116257</v>
+        <v>116456</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11361</v>
+        <v>11381</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+199⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1215,11 +1215,11 @@
         <v>95579</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9571</v>
+        <v>9573</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>87690</v>
+        <v>87790</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11489</v>
+        <v>11499</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+135⭐)</t>
+          <t>📈 Trending (+100⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1284,7 +1284,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -1298,14 +1298,14 @@
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>80301</v>
+        <v>80302</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>6102</v>
+        <v>6105</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+14⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>212619</v>
+        <v>212797</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21552</v>
+        <v>21567</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+225⭐)</t>
+          <t>📈 Trending (+178⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187289</v>
+        <v>187313</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46019</v>
+        <v>46016</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+19⭐)</t>
+          <t>📈 Trending (+24⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>180761</v>
+        <v>180838</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17833</v>
+        <v>17840</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+62⭐)</t>
+          <t>📈 Trending (+77⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>179607</v>
+        <v>180017</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9766</v>
+        <v>9781</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-15]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>245183</v>
+        <v>245539</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>51004</v>
+        <v>51156</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>155628</v>
+        <v>155738</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24577</v>
+        <v>24597</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+74⭐)</t>
+          <t>📈 Trending (+110⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>154748</v>
+        <v>154806</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10083</v>
+        <v>10088</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+69⭐)</t>
+          <t>📈 Trending (+58⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>152151</v>
+        <v>152357</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24513</v>
+        <v>24551</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+209⭐)</t>
+          <t>📈 Trending (+206⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143603</v>
+        <v>143632</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34812</v>
+        <v>34810</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+31⭐)</t>
+          <t>📈 Trending (+29⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49110</v>
+        <v>49134</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4867</v>
+        <v>4872</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+30⭐)</t>
+          <t>📈 Trending (+24⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13726</v>
+        <v>13761</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1640</v>
+        <v>1644</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+13⭐)</t>
+          <t>📈 Trending (+35⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10955</v>
+        <v>10957</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2603</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+5⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5704</v>
+        <v>5706</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>713</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>257785</v>
+        <v>258427</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>38552</v>
+        <v>38655</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,14 +1126,14 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>137393</v>
+        <v>138490</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7381</v>
+        <v>7437</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>116456</v>
+        <v>116758</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11381</v>
+        <v>11398</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+199⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1215,7 +1215,7 @@
         <v>95579</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9573</v>
+        <v>9578</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>87790</v>
+        <v>87926</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11499</v>
+        <v>11525</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+100⭐)</t>
+          <t>📈 Trending (+136⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>212797</v>
+        <v>213024</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21567</v>
+        <v>21581</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+178⭐)</t>
+          <t>📈 Trending (+227⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187313</v>
+        <v>187344</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>46016</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+24⭐)</t>
+          <t>📈 Trending (+31⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>180838</v>
+        <v>180967</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17840</v>
+        <v>17871</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+77⭐)</t>
+          <t>📈 Trending (+129⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Get up and running with Kimi-K2.6, GLM-5.2, MiniMax, DeepSeek, gpt-oss, Qwen, Gemma and other models.</t>
+          <t>Get up and running with Kimi, GLM, MiniMax, DeepSeek, gpt-oss, Qwen, Gemma and other models.</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>180017</v>
+        <v>180456</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9781</v>
+        <v>9790</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1493,6 +1493,59 @@
       <c r="I24" s="7" t="inlineStr">
         <is>
           <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>🛠️ Developer Tools &amp; Powerful CLIs</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>rtk-ai/rtk</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>80397</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>5100</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>✨ Featured</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Rust</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>CLI proxy that reduces LLM token consumption by 60-90% on common dev commands. Single Rust binary, zero dependencies</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>agentic-coding, ai-coding, anthropic, claude-code, cli</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/rtk-ai/rtk</t>
         </is>
       </c>
     </row>
@@ -1520,6 +1573,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-16]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>245539</v>
+        <v>245889</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>51156</v>
+        <v>51314</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>155738</v>
+        <v>155868</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24597</v>
+        <v>24618</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+110⭐)</t>
+          <t>📈 Trending (+130⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>154806</v>
+        <v>154852</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10088</v>
+        <v>10099</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+58⭐)</t>
+          <t>📈 Trending (+46⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>152357</v>
+        <v>152605</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24551</v>
+        <v>24599</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+206⭐)</t>
+          <t>📈 Trending (+248⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143632</v>
+        <v>143654</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34810</v>
+        <v>34815</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+29⭐)</t>
+          <t>📈 Trending (+22⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49134</v>
+        <v>49166</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4872</v>
+        <v>4876</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+24⭐)</t>
+          <t>📈 Trending (+32⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13761</v>
+        <v>13777</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1644</v>
+        <v>1646</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+35⭐)</t>
+          <t>📈 Trending (+16⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10957</v>
+        <v>10958</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2603</v>
+        <v>2604</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5706</v>
+        <v>5708</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>713</v>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>258427</v>
+        <v>259360</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>38655</v>
+        <v>38798</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>138490</v>
+        <v>139426</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7437</v>
+        <v>7489</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>116758</v>
+        <v>118062</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11398</v>
+        <v>11411</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>🔥 Supernova (+1000⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95579</v>
+        <v>95581</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9578</v>
+        <v>9576</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>87926</v>
+        <v>88050</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11525</v>
+        <v>11549</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+136⭐)</t>
+          <t>📈 Trending (+124⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>213024</v>
+        <v>213227</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21581</v>
+        <v>21601</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+227⭐)</t>
+          <t>📈 Trending (+203⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187344</v>
+        <v>187368</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46016</v>
+        <v>46012</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+31⭐)</t>
+          <t>📈 Trending (+24⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>180967</v>
+        <v>181079</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17871</v>
+        <v>17892</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+129⭐)</t>
+          <t>📈 Trending (+112⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>180456</v>
+        <v>180907</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9790</v>
+        <v>9810</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>80397</v>
+        <v>80588</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5100</v>
+        <v>5109</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+191⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-17]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>245889</v>
+        <v>246214</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>51314</v>
+        <v>51480</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>155868</v>
+        <v>156023</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24618</v>
+        <v>24637</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+130⭐)</t>
+          <t>📈 Trending (+155⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,10 +653,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>154852</v>
+        <v>154898</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10099</v>
+        <v>10107</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>152605</v>
+        <v>152928</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24599</v>
+        <v>24664</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+248⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143654</v>
+        <v>143679</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34815</v>
+        <v>34818</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+22⭐)</t>
+          <t>📈 Trending (+25⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49166</v>
+        <v>49196</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4876</v>
+        <v>4884</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+32⭐)</t>
+          <t>📈 Trending (+30⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13777</v>
+        <v>13786</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1646</v>
+        <v>1648</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+16⭐)</t>
+          <t>📈 Trending (+9⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10958</v>
+        <v>10959</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2604</v>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6235</v>
+        <v>6233</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>301</v>
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5708</v>
+        <v>5707</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>713</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>259360</v>
+        <v>260335</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>38798</v>
+        <v>38966</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>139426</v>
+        <v>140419</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7489</v>
+        <v>7543</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>118062</v>
+        <v>118482</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11411</v>
+        <v>11460</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>🔥 Supernova (+1000⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95581</v>
+        <v>95586</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>9576</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+5⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>88050</v>
+        <v>88198</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11549</v>
+        <v>11579</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+124⭐)</t>
+          <t>📈 Trending (+148⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>213227</v>
+        <v>213462</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21601</v>
+        <v>21611</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+203⭐)</t>
+          <t>📈 Trending (+235⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187368</v>
+        <v>187394</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46012</v>
+        <v>46014</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+24⭐)</t>
+          <t>📈 Trending (+26⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181079</v>
+        <v>181194</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17892</v>
+        <v>17912</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+112⭐)</t>
+          <t>📈 Trending (+115⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>180907</v>
+        <v>181331</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9810</v>
+        <v>9828</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>The context API to search, scrape, and interact with the web at scale. 🔥</t>
+          <t>The web data API to search, scrape, and interact at scale. 🔥</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>80588</v>
+        <v>80751</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5109</v>
+        <v>5112</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+191⭐)</t>
+          <t>📈 Trending (+163⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-18]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>246214</v>
+        <v>246570</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>51480</v>
+        <v>51652</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>156023</v>
+        <v>156196</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24637</v>
+        <v>24667</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+155⭐)</t>
+          <t>📈 Trending (+173⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>154898</v>
+        <v>154950</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10107</v>
+        <v>10109</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+46⭐)</t>
+          <t>📈 Trending (+52⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>152928</v>
+        <v>153189</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24664</v>
+        <v>24713</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+261⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,10 +739,10 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143679</v>
+        <v>143704</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34818</v>
+        <v>34820</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49196</v>
+        <v>49229</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4884</v>
+        <v>4892</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+30⭐)</t>
+          <t>📈 Trending (+33⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13786</v>
+        <v>13807</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1648</v>
+        <v>1652</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+9⭐)</t>
+          <t>📈 Trending (+21⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10959</v>
+        <v>10961</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2604</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5707</v>
+        <v>5708</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>713</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>260335</v>
+        <v>261203</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>38966</v>
+        <v>39103</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>140419</v>
+        <v>141367</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7543</v>
+        <v>7579</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>118482</v>
+        <v>119090</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11460</v>
+        <v>11515</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+5⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>88198</v>
+        <v>88342</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11579</v>
+        <v>11605</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+148⭐)</t>
+          <t>📈 Trending (+144⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>213462</v>
+        <v>213733</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21611</v>
+        <v>21630</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+235⭐)</t>
+          <t>📈 Trending (+271⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187394</v>
+        <v>187418</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46014</v>
+        <v>46007</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+26⭐)</t>
+          <t>📈 Trending (+24⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181194</v>
+        <v>181177</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17912</v>
+        <v>17920</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+115⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>181331</v>
+        <v>181704</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9828</v>
+        <v>9838</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>80751</v>
+        <v>80845</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5112</v>
+        <v>5123</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+163⭐)</t>
+          <t>📈 Trending (+94⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-19]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>246570</v>
+        <v>246927</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>51652</v>
+        <v>51803</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>156196</v>
+        <v>156361</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24667</v>
+        <v>24681</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+173⭐)</t>
+          <t>📈 Trending (+165⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>154950</v>
+        <v>154992</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10109</v>
+        <v>10113</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+52⭐)</t>
+          <t>📈 Trending (+42⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>153189</v>
+        <v>153400</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24713</v>
+        <v>24743</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+261⭐)</t>
+          <t>📈 Trending (+211⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143704</v>
+        <v>143709</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34820</v>
+        <v>34816</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+25⭐)</t>
+          <t>📈 Trending (+5⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49229</v>
+        <v>49252</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>4892</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+33⭐)</t>
+          <t>📈 Trending (+23⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13807</v>
+        <v>13819</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1652</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+21⭐)</t>
+          <t>📈 Trending (+12⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10961</v>
+        <v>10962</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2604</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6233</v>
+        <v>6235</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>301</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5708</v>
+        <v>5710</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>713</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>3875</v>
+        <v>3874</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>466</v>
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>261203</v>
+        <v>262102</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>39103</v>
+        <v>39220</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>141367</v>
+        <v>142046</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7579</v>
+        <v>7616</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>119090</v>
+        <v>119396</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11515</v>
+        <v>11542</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95586</v>
+        <v>95592</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>9576</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+6⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>88342</v>
+        <v>88454</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11605</v>
+        <v>11618</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+144⭐)</t>
+          <t>📈 Trending (+112⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>213733</v>
+        <v>213984</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21630</v>
+        <v>21641</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+271⭐)</t>
+          <t>📈 Trending (+251⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187418</v>
+        <v>187440</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46007</v>
+        <v>46004</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+24⭐)</t>
+          <t>📈 Trending (+22⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181177</v>
+        <v>181234</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17920</v>
+        <v>17924</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+57⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>181704</v>
+        <v>182023</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9838</v>
+        <v>9846</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>80845</v>
+        <v>80950</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5123</v>
+        <v>5135</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+94⭐)</t>
+          <t>📈 Trending (+105⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-20]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>246927</v>
+        <v>247173</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>51803</v>
+        <v>51937</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>156361</v>
+        <v>156493</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24681</v>
+        <v>24689</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+165⭐)</t>
+          <t>📈 Trending (+132⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>154992</v>
+        <v>155023</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10113</v>
+        <v>10119</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+42⭐)</t>
+          <t>📈 Trending (+31⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>153400</v>
+        <v>153561</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24743</v>
+        <v>24766</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+211⭐)</t>
+          <t>📈 Trending (+161⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143709</v>
+        <v>143738</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34816</v>
+        <v>34808</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+5⭐)</t>
+          <t>📈 Trending (+29⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49252</v>
+        <v>49271</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4892</v>
+        <v>4894</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+23⭐)</t>
+          <t>📈 Trending (+19⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13819</v>
+        <v>13837</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1652</v>
+        <v>1653</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+12⭐)</t>
+          <t>📈 Trending (+18⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,10 +911,10 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10962</v>
+        <v>10963</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2604</v>
+        <v>2603</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6235</v>
+        <v>6236</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>301</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>262102</v>
+        <v>262988</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>39220</v>
+        <v>39352</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>142046</v>
+        <v>142559</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7616</v>
+        <v>7651</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>119396</v>
+        <v>119655</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11542</v>
+        <v>11566</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+259⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95592</v>
+        <v>95591</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9576</v>
+        <v>9579</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+6⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>88454</v>
+        <v>88551</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11618</v>
+        <v>11635</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+112⭐)</t>
+          <t>📈 Trending (+97⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>213984</v>
+        <v>214149</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21641</v>
+        <v>21660</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+251⭐)</t>
+          <t>📈 Trending (+165⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187440</v>
+        <v>187449</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46004</v>
+        <v>46007</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+22⭐)</t>
+          <t>📈 Trending (+9⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181234</v>
+        <v>181283</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17924</v>
+        <v>17939</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+57⭐)</t>
+          <t>📈 Trending (+49⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,14 +1470,14 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>182023</v>
+        <v>182305</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9846</v>
+        <v>9853</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+282⭐)</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>80950</v>
+        <v>81053</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5135</v>
+        <v>5137</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+105⭐)</t>
+          <t>📈 Trending (+103⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-21]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>247173</v>
+        <v>247489</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>51937</v>
+        <v>52064</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>156493</v>
+        <v>156640</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24689</v>
+        <v>24699</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+132⭐)</t>
+          <t>📈 Trending (+147⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155023</v>
+        <v>155060</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10119</v>
+        <v>10120</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+31⭐)</t>
+          <t>📈 Trending (+37⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>153561</v>
+        <v>153781</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24766</v>
+        <v>24807</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+161⭐)</t>
+          <t>📈 Trending (+220⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143738</v>
+        <v>143755</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34808</v>
+        <v>34811</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+29⭐)</t>
+          <t>📈 Trending (+17⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49271</v>
+        <v>49293</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4894</v>
+        <v>4896</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+19⭐)</t>
+          <t>📈 Trending (+22⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13837</v>
+        <v>13855</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1653</v>
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10963</v>
+        <v>10964</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2603</v>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,10 +997,10 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5710</v>
+        <v>5708</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>262988</v>
+        <v>263799</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>39352</v>
+        <v>39463</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>142559</v>
+        <v>143111</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7651</v>
+        <v>7674</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>119655</v>
+        <v>119917</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11566</v>
+        <v>11593</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+259⭐)</t>
+          <t>📈 Trending (+262⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95591</v>
+        <v>95598</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9579</v>
+        <v>9580</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+7⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>88551</v>
+        <v>88655</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11635</v>
+        <v>11664</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+97⭐)</t>
+          <t>📈 Trending (+104⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>214149</v>
+        <v>214353</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21660</v>
+        <v>21672</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+165⭐)</t>
+          <t>📈 Trending (+204⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187449</v>
+        <v>187466</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46007</v>
+        <v>46006</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+9⭐)</t>
+          <t>📈 Trending (+17⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181283</v>
+        <v>181331</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17939</v>
+        <v>17946</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+49⭐)</t>
+          <t>📈 Trending (+48⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,14 +1470,14 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>182305</v>
+        <v>182614</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9853</v>
+        <v>9867</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+282⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>81053</v>
+        <v>81159</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5137</v>
+        <v>5144</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+103⭐)</t>
+          <t>📈 Trending (+106⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-22]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>247489</v>
+        <v>247798</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>52064</v>
+        <v>52198</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>156640</v>
+        <v>156780</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24699</v>
+        <v>24722</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+147⭐)</t>
+          <t>📈 Trending (+140⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155060</v>
+        <v>155108</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10120</v>
+        <v>10122</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+37⭐)</t>
+          <t>📈 Trending (+48⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>153781</v>
+        <v>154003</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24807</v>
+        <v>24850</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+220⭐)</t>
+          <t>📈 Trending (+222⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143755</v>
+        <v>143777</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34811</v>
+        <v>34809</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+17⭐)</t>
+          <t>📈 Trending (+22⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49293</v>
+        <v>49316</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4896</v>
+        <v>4904</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+22⭐)</t>
+          <t>📈 Trending (+23⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13855</v>
+        <v>13866</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+18⭐)</t>
+          <t>📈 Trending (+11⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10964</v>
+        <v>10966</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2603</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6236</v>
+        <v>6237</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>301</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5708</v>
+        <v>5709</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>712</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>263799</v>
+        <v>264777</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>39463</v>
+        <v>39567</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>143111</v>
+        <v>143766</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7674</v>
+        <v>7700</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>119917</v>
+        <v>120228</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11593</v>
+        <v>11607</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+262⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95598</v>
+        <v>95607</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9580</v>
+        <v>9579</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+7⭐)</t>
+          <t>📈 Trending (+9⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>88655</v>
+        <v>88752</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11664</v>
+        <v>11675</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+104⭐)</t>
+          <t>📈 Trending (+97⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>214353</v>
+        <v>214521</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21672</v>
+        <v>21687</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+204⭐)</t>
+          <t>📈 Trending (+168⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,10 +1384,10 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187466</v>
+        <v>187483</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46006</v>
+        <v>46007</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181331</v>
+        <v>181415</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17946</v>
+        <v>17963</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+48⭐)</t>
+          <t>📈 Trending (+84⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>182614</v>
+        <v>182997</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9867</v>
+        <v>9880</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>81159</v>
+        <v>81329</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5144</v>
+        <v>5153</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+106⭐)</t>
+          <t>📈 Trending (+170⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-23]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>247798</v>
+        <v>248125</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>52198</v>
+        <v>52362</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>156780</v>
+        <v>156893</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24722</v>
+        <v>24733</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+140⭐)</t>
+          <t>📈 Trending (+113⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155108</v>
+        <v>155150</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10122</v>
+        <v>10127</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+48⭐)</t>
+          <t>📈 Trending (+42⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>154003</v>
+        <v>154207</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24850</v>
+        <v>24883</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+222⭐)</t>
+          <t>📈 Trending (+204⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143777</v>
+        <v>143817</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34809</v>
+        <v>34810</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+22⭐)</t>
+          <t>📈 Trending (+40⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49316</v>
+        <v>49339</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4904</v>
+        <v>4905</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13866</v>
+        <v>13881</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1654</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+11⭐)</t>
+          <t>📈 Trending (+15⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,10 +911,10 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10966</v>
+        <v>10968</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2603</v>
+        <v>2602</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -957,11 +957,11 @@
         <v>6237</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5709</v>
+        <v>5710</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>712</v>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>264777</v>
+        <v>265489</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>39567</v>
+        <v>39672</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>143766</v>
+        <v>144469</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7700</v>
+        <v>7733</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>120228</v>
+        <v>120592</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11607</v>
+        <v>11638</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95607</v>
+        <v>95612</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9579</v>
+        <v>9578</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+9⭐)</t>
+          <t>📈 Trending (+5⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>88752</v>
+        <v>88883</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11675</v>
+        <v>11695</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+97⭐)</t>
+          <t>📈 Trending (+131⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>214521</v>
+        <v>214668</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21687</v>
+        <v>21696</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+168⭐)</t>
+          <t>📈 Trending (+147⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187483</v>
+        <v>187503</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46007</v>
+        <v>46002</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+17⭐)</t>
+          <t>📈 Trending (+20⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181415</v>
+        <v>181493</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17963</v>
+        <v>17974</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+84⭐)</t>
+          <t>📈 Trending (+78⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>182997</v>
+        <v>183453</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9880</v>
+        <v>9889</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>81329</v>
+        <v>81458</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5153</v>
+        <v>5158</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+170⭐)</t>
+          <t>📈 Trending (+129⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-24]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>248125</v>
+        <v>248423</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>52362</v>
+        <v>52513</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>156893</v>
+        <v>157009</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24733</v>
+        <v>24740</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+113⭐)</t>
+          <t>📈 Trending (+116⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155150</v>
+        <v>155191</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10127</v>
+        <v>10130</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+42⭐)</t>
+          <t>📈 Trending (+41⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>154207</v>
+        <v>154386</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24883</v>
+        <v>24910</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+204⭐)</t>
+          <t>📈 Trending (+179⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143817</v>
+        <v>143834</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34810</v>
+        <v>34816</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+40⭐)</t>
+          <t>📈 Trending (+17⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49339</v>
+        <v>49362</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4905</v>
+        <v>4907</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,10 +868,10 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13881</v>
+        <v>13896</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10968</v>
+        <v>10969</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2602</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5710</v>
+        <v>5711</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>712</v>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>265489</v>
+        <v>266209</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>39672</v>
+        <v>39782</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>144469</v>
+        <v>145043</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7733</v>
+        <v>7774</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>120592</v>
+        <v>120932</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11638</v>
+        <v>11662</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,10 +1212,10 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95612</v>
+        <v>95617</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9578</v>
+        <v>9581</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>88883</v>
+        <v>88998</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11695</v>
+        <v>11715</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+131⭐)</t>
+          <t>📈 Trending (+115⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>214668</v>
+        <v>214840</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21696</v>
+        <v>21707</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+147⭐)</t>
+          <t>📈 Trending (+172⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187503</v>
+        <v>187515</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>46002</v>
+        <v>45997</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+20⭐)</t>
+          <t>📈 Trending (+12⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181493</v>
+        <v>181538</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17974</v>
+        <v>17983</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+78⭐)</t>
+          <t>📈 Trending (+45⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>183453</v>
+        <v>183892</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9889</v>
+        <v>9904</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>81458</v>
+        <v>81591</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5158</v>
+        <v>5161</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+129⭐)</t>
+          <t>📈 Trending (+133⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-25]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>248423</v>
+        <v>248744</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>52513</v>
+        <v>52653</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157009</v>
+        <v>157126</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24740</v>
+        <v>24771</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+116⭐)</t>
+          <t>📈 Trending (+117⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155191</v>
+        <v>155223</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10130</v>
+        <v>10142</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+41⭐)</t>
+          <t>📈 Trending (+32⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>154386</v>
+        <v>154533</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24910</v>
+        <v>24938</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+179⭐)</t>
+          <t>📈 Trending (+147⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143834</v>
+        <v>143848</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34816</v>
+        <v>34815</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+17⭐)</t>
+          <t>📈 Trending (+14⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49362</v>
+        <v>49377</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4907</v>
+        <v>4912</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+23⭐)</t>
+          <t>📈 Trending (+15⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13896</v>
+        <v>13903</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1655</v>
+        <v>1657</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+15⭐)</t>
+          <t>📈 Trending (+7⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -914,11 +914,11 @@
         <v>10969</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2602</v>
+        <v>2603</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6237</v>
+        <v>6238</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5711</v>
+        <v>5712</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>712</v>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>266209</v>
+        <v>266944</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>39782</v>
+        <v>39891</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>145043</v>
+        <v>145573</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7774</v>
+        <v>7803</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>120932</v>
+        <v>121225</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11662</v>
+        <v>11686</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+293⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95617</v>
+        <v>95618</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9581</v>
+        <v>9580</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+5⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>88998</v>
+        <v>89102</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11715</v>
+        <v>11732</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+115⭐)</t>
+          <t>📈 Trending (+104⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>214840</v>
+        <v>215017</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21707</v>
+        <v>21725</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+172⭐)</t>
+          <t>📈 Trending (+177⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187515</v>
+        <v>187536</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>45997</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+12⭐)</t>
+          <t>📈 Trending (+21⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181538</v>
+        <v>181652</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17983</v>
+        <v>17999</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+45⭐)</t>
+          <t>📈 Trending (+114⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>183892</v>
+        <v>184344</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9904</v>
+        <v>9912</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>81591</v>
+        <v>81663</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5161</v>
+        <v>5167</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+133⭐)</t>
+          <t>📈 Trending (+72⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-26]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>248744</v>
+        <v>248990</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>52653</v>
+        <v>52812</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157126</v>
+        <v>157223</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24771</v>
+        <v>24781</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+117⭐)</t>
+          <t>📈 Trending (+97⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155223</v>
+        <v>155264</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10142</v>
+        <v>10147</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+32⭐)</t>
+          <t>📈 Trending (+41⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>154533</v>
+        <v>154653</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24938</v>
+        <v>24949</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+147⭐)</t>
+          <t>📈 Trending (+120⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143848</v>
+        <v>143876</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34815</v>
+        <v>34810</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+14⭐)</t>
+          <t>📈 Trending (+28⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49377</v>
+        <v>49408</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4912</v>
+        <v>4915</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+15⭐)</t>
+          <t>📈 Trending (+31⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13903</v>
+        <v>13916</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1657</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+7⭐)</t>
+          <t>📈 Trending (+13⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10969</v>
+        <v>10970</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2603</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5712</v>
+        <v>5713</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>712</v>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>266944</v>
+        <v>267535</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>39891</v>
+        <v>39963</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>145573</v>
+        <v>146019</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7803</v>
+        <v>7834</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>121225</v>
+        <v>121464</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11686</v>
+        <v>11704</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+293⭐)</t>
+          <t>📈 Trending (+239⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95618</v>
+        <v>95622</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9580</v>
+        <v>9579</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>89102</v>
+        <v>89172</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11732</v>
+        <v>11744</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+104⭐)</t>
+          <t>📈 Trending (+70⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>215017</v>
+        <v>215172</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21725</v>
+        <v>21735</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+177⭐)</t>
+          <t>📈 Trending (+155⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187536</v>
+        <v>187564</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45997</v>
+        <v>45996</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+21⭐)</t>
+          <t>📈 Trending (+28⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181652</v>
+        <v>181733</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17999</v>
+        <v>18006</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+114⭐)</t>
+          <t>📈 Trending (+81⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>184344</v>
+        <v>184763</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9912</v>
+        <v>9926</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>81663</v>
+        <v>81726</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5167</v>
+        <v>5180</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+72⭐)</t>
+          <t>📈 Trending (+63⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-27]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>248990</v>
+        <v>249253</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>52812</v>
+        <v>52936</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157223</v>
+        <v>157290</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24781</v>
+        <v>24792</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+97⭐)</t>
+          <t>📈 Trending (+67⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155264</v>
+        <v>155286</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10147</v>
+        <v>10149</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+41⭐)</t>
+          <t>📈 Trending (+22⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>154653</v>
+        <v>154780</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24949</v>
+        <v>24960</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+120⭐)</t>
+          <t>📈 Trending (+127⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143876</v>
+        <v>143887</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>34810</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+28⭐)</t>
+          <t>📈 Trending (+11⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49408</v>
+        <v>49430</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4915</v>
+        <v>4918</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+31⭐)</t>
+          <t>📈 Trending (+22⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13916</v>
+        <v>13926</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1657</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+13⭐)</t>
+          <t>📈 Trending (+10⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10970</v>
+        <v>10972</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2603</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>267535</v>
+        <v>267985</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>39963</v>
+        <v>40029</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>146019</v>
+        <v>146534</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7834</v>
+        <v>7877</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>121464</v>
+        <v>121679</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11704</v>
+        <v>11712</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+239⭐)</t>
+          <t>📈 Trending (+215⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1215,11 +1215,11 @@
         <v>95622</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9579</v>
+        <v>9584</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+4⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>89172</v>
+        <v>89241</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11744</v>
+        <v>11759</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+70⭐)</t>
+          <t>📈 Trending (+69⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>215172</v>
+        <v>215379</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21735</v>
+        <v>21745</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+155⭐)</t>
+          <t>📈 Trending (+207⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187564</v>
+        <v>187583</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45996</v>
+        <v>45990</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+28⭐)</t>
+          <t>📈 Trending (+19⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181733</v>
+        <v>181778</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18006</v>
+        <v>18016</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+81⭐)</t>
+          <t>📈 Trending (+45⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>184763</v>
+        <v>185161</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9926</v>
+        <v>9934</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>81726</v>
+        <v>81775</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5180</v>
+        <v>5185</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+63⭐)</t>
+          <t>📈 Trending (+49⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-28]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>249253</v>
+        <v>249518</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>52936</v>
+        <v>53065</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157290</v>
+        <v>157352</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24792</v>
+        <v>24798</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+67⭐)</t>
+          <t>📈 Trending (+62⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155286</v>
+        <v>155313</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10149</v>
+        <v>10148</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+22⭐)</t>
+          <t>📈 Trending (+27⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>154780</v>
+        <v>154925</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24960</v>
+        <v>24984</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+127⭐)</t>
+          <t>📈 Trending (+145⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143887</v>
+        <v>143907</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>34810</v>
+        <v>34803</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+11⭐)</t>
+          <t>📈 Trending (+20⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49430</v>
+        <v>49516</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4918</v>
+        <v>4931</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+22⭐)</t>
+          <t>📈 Trending (+86⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13926</v>
+        <v>13935</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1657</v>
+        <v>1663</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+10⭐)</t>
+          <t>📈 Trending (+9⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10972</v>
+        <v>10971</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2603</v>
+        <v>2602</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6238</v>
+        <v>6237</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>267985</v>
+        <v>268452</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>40029</v>
+        <v>40107</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>146534</v>
+        <v>146956</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7877</v>
+        <v>7896</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>121679</v>
+        <v>121894</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11712</v>
+        <v>11742</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95622</v>
+        <v>95625</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>9584</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>89241</v>
+        <v>89321</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11759</v>
+        <v>11771</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+69⭐)</t>
+          <t>📈 Trending (+80⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>215379</v>
+        <v>215552</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21745</v>
+        <v>21760</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+207⭐)</t>
+          <t>📈 Trending (+173⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187583</v>
+        <v>187594</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45990</v>
+        <v>45981</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+19⭐)</t>
+          <t>📈 Trending (+11⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181778</v>
+        <v>181820</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18016</v>
+        <v>18026</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+45⭐)</t>
+          <t>📈 Trending (+42⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>185161</v>
+        <v>185577</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9934</v>
+        <v>9951</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>81775</v>
+        <v>81837</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5185</v>
+        <v>5190</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+49⭐)</t>
+          <t>📈 Trending (+62⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-29]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>249518</v>
+        <v>249828</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>53065</v>
+        <v>53242</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157352</v>
+        <v>157438</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24798</v>
+        <v>24807</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+62⭐)</t>
+          <t>📈 Trending (+86⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155313</v>
+        <v>155342</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10148</v>
+        <v>10150</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+27⭐)</t>
+          <t>📈 Trending (+29⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>154925</v>
+        <v>155129</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>24984</v>
+        <v>25024</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+145⭐)</t>
+          <t>📈 Trending (+204⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -739,14 +739,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>143907</v>
+        <v>143923</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>34803</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+20⭐)</t>
+          <t>📈 Trending (+16⭐)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49516</v>
+        <v>49745</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4931</v>
+        <v>4953</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+86⭐)</t>
+          <t>📈 Trending (+229⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13935</v>
+        <v>13941</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1663</v>
+        <v>1666</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+9⭐)</t>
+          <t>📈 Trending (+6⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10971</v>
+        <v>10970</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2602</v>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5713</v>
+        <v>5716</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>712</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>268452</v>
+        <v>269064</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>40107</v>
+        <v>40204</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>146956</v>
+        <v>147606</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7896</v>
+        <v>7929</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>121894</v>
+        <v>122178</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11742</v>
+        <v>11771</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+215⭐)</t>
+          <t>📈 Trending (+284⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95625</v>
+        <v>95635</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9584</v>
+        <v>9585</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>📈 Trending (+10⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>89321</v>
+        <v>89422</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11771</v>
+        <v>11792</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+80⭐)</t>
+          <t>📈 Trending (+101⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>215552</v>
+        <v>215721</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21760</v>
+        <v>21761</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+173⭐)</t>
+          <t>📈 Trending (+169⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187594</v>
+        <v>187596</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>45981</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+11⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181820</v>
+        <v>181878</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18026</v>
+        <v>18037</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+42⭐)</t>
+          <t>📈 Trending (+58⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>185577</v>
+        <v>186073</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9951</v>
+        <v>9966</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>81837</v>
+        <v>81936</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5190</v>
+        <v>5199</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+62⭐)</t>
+          <t>📈 Trending (+99⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-09-30]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>249828</v>
+        <v>250099</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>53242</v>
+        <v>53392</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157438</v>
+        <v>157532</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24807</v>
+        <v>24830</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+86⭐)</t>
+          <t>📈 Trending (+94⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155342</v>
+        <v>155381</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10150</v>
+        <v>10144</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+29⭐)</t>
+          <t>📈 Trending (+39⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>155129</v>
+        <v>155353</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25024</v>
+        <v>25063</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+204⭐)</t>
+          <t>📈 Trending (+224⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49745</v>
+        <v>49836</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4953</v>
+        <v>4968</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+229⭐)</t>
+          <t>📈 Trending (+91⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13941</v>
+        <v>13956</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1666</v>
+        <v>1668</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+6⭐)</t>
+          <t>📈 Trending (+15⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6237</v>
+        <v>6236</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,10 +997,10 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5716</v>
+        <v>5719</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>269064</v>
+        <v>269683</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>40204</v>
+        <v>40295</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>147606</v>
+        <v>148283</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7929</v>
+        <v>7974</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>122178</v>
+        <v>122502</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11771</v>
+        <v>11805</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+284⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95635</v>
+        <v>95639</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9585</v>
+        <v>9584</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+10⭐)</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>89422</v>
+        <v>89553</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11792</v>
+        <v>11817</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+101⭐)</t>
+          <t>📈 Trending (+131⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>215721</v>
+        <v>215907</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21761</v>
+        <v>21780</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+169⭐)</t>
+          <t>📈 Trending (+186⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187596</v>
+        <v>187621</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45981</v>
+        <v>45980</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+25⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181878</v>
+        <v>181934</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18037</v>
+        <v>18042</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+58⭐)</t>
+          <t>📈 Trending (+56⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,14 +1470,14 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>186073</v>
+        <v>186693</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9966</v>
+        <v>9984</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>The web data API to search, scrape, and interact at scale. 🔥</t>
+          <t>🔥 Supercharge your AI agents with data from the web and beyond. A web data API to search, scrape, and access more sources.</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>81936</v>
+        <v>82037</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5199</v>
+        <v>5203</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+99⭐)</t>
+          <t>📈 Trending (+101⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-01]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>250099</v>
+        <v>250370</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>53392</v>
+        <v>53506</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157532</v>
+        <v>157623</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24830</v>
+        <v>24862</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+94⭐)</t>
+          <t>📈 Trending (+91⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155381</v>
+        <v>155406</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10144</v>
+        <v>10155</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+39⭐)</t>
+          <t>📈 Trending (+25⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>155353</v>
+        <v>155541</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25063</v>
+        <v>25101</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+224⭐)</t>
+          <t>📈 Trending (+188⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49836</v>
+        <v>49896</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4968</v>
+        <v>4977</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+91⭐)</t>
+          <t>📈 Trending (+60⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13956</v>
+        <v>13963</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1668</v>
+        <v>1667</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+15⭐)</t>
+          <t>📈 Trending (+7⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -914,7 +914,7 @@
         <v>10970</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2602</v>
+        <v>2601</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6236</v>
+        <v>6237</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>269683</v>
+        <v>270243</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>40295</v>
+        <v>40392</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>148283</v>
+        <v>149261</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>7974</v>
+        <v>8023</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>122502</v>
+        <v>122837</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11805</v>
+        <v>11837</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95639</v>
+        <v>95643</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>9584</v>
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>89553</v>
+        <v>89660</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11817</v>
+        <v>11837</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+131⭐)</t>
+          <t>📈 Trending (+107⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>215907</v>
+        <v>216064</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21780</v>
+        <v>21803</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+186⭐)</t>
+          <t>📈 Trending (+157⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187621</v>
+        <v>187630</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>45980</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+25⭐)</t>
+          <t>📈 Trending (+9⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181934</v>
+        <v>181980</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18042</v>
+        <v>18057</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+56⭐)</t>
+          <t>📈 Trending (+46⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>186693</v>
+        <v>187213</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9984</v>
+        <v>9994</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>82037</v>
+        <v>82122</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5203</v>
+        <v>5212</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+101⭐)</t>
+          <t>📈 Trending (+85⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-02]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>250370</v>
+        <v>250623</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>53506</v>
+        <v>53652</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157623</v>
+        <v>157702</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24862</v>
+        <v>24880</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+91⭐)</t>
+          <t>📈 Trending (+79⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155406</v>
+        <v>155444</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10155</v>
+        <v>10162</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+25⭐)</t>
+          <t>📈 Trending (+38⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>155541</v>
+        <v>155640</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25101</v>
+        <v>25133</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+188⭐)</t>
+          <t>📈 Trending (+99⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49896</v>
+        <v>49922</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4977</v>
+        <v>4982</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+60⭐)</t>
+          <t>📈 Trending (+26⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13963</v>
+        <v>13965</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1667</v>
+        <v>1669</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+7⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10970</v>
+        <v>10972</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2601</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6237</v>
+        <v>6238</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>270243</v>
+        <v>270744</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>40392</v>
+        <v>40474</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>149261</v>
+        <v>150618</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8023</v>
+        <v>8086</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>122837</v>
+        <v>123108</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11837</v>
+        <v>11868</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+271⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95643</v>
+        <v>95645</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9584</v>
+        <v>9586</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+4⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>89660</v>
+        <v>89758</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11837</v>
+        <v>11855</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+107⭐)</t>
+          <t>📈 Trending (+98⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>216064</v>
+        <v>216250</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21803</v>
+        <v>21808</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+157⭐)</t>
+          <t>📈 Trending (+186⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187630</v>
+        <v>187650</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45980</v>
+        <v>45974</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+9⭐)</t>
+          <t>📈 Trending (+20⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>181980</v>
+        <v>182029</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18057</v>
+        <v>18075</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+46⭐)</t>
+          <t>📈 Trending (+49⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>187213</v>
+        <v>187621</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>9994</v>
+        <v>10009</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>82122</v>
+        <v>82182</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5212</v>
+        <v>5213</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+85⭐)</t>
+          <t>📈 Trending (+60⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-03]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>250623</v>
+        <v>250790</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>53652</v>
+        <v>53737</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157702</v>
+        <v>157733</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24880</v>
+        <v>24891</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+79⭐)</t>
+          <t>📈 Trending (+31⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155444</v>
+        <v>155460</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10162</v>
+        <v>10169</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+38⭐)</t>
+          <t>📈 Trending (+16⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>155640</v>
+        <v>155828</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25133</v>
+        <v>25138</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+99⭐)</t>
+          <t>📈 Trending (+188⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49922</v>
+        <v>49943</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4982</v>
+        <v>4980</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+26⭐)</t>
+          <t>📈 Trending (+21⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13965</v>
+        <v>13971</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1669</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+6⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10972</v>
+        <v>10975</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2601</v>
+        <v>2600</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6238</v>
+        <v>6239</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>270744</v>
+        <v>271405</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>40474</v>
+        <v>40545</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>150618</v>
+        <v>151885</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8086</v>
+        <v>8145</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>123108</v>
+        <v>123353</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11868</v>
+        <v>11888</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+271⭐)</t>
+          <t>📈 Trending (+245⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95645</v>
+        <v>95644</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>9586</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>89758</v>
+        <v>89828</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11855</v>
+        <v>11864</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+98⭐)</t>
+          <t>📈 Trending (+70⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>216250</v>
+        <v>216595</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21808</v>
+        <v>21810</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+186⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187650</v>
+        <v>187639</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45974</v>
+        <v>45959</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+20⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>182029</v>
+        <v>182069</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18075</v>
+        <v>18085</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+49⭐)</t>
+          <t>📈 Trending (+40⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>187621</v>
+        <v>187981</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10009</v>
+        <v>10008</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>82182</v>
+        <v>82255</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5213</v>
+        <v>5223</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+60⭐)</t>
+          <t>📈 Trending (+73⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-04]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>250790</v>
+        <v>251001</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>53737</v>
+        <v>53828</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157733</v>
+        <v>157788</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24891</v>
+        <v>24899</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+31⭐)</t>
+          <t>📈 Trending (+55⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155460</v>
+        <v>155488</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10169</v>
+        <v>10175</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+16⭐)</t>
+          <t>📈 Trending (+28⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>155828</v>
+        <v>156041</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25138</v>
+        <v>25176</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+188⭐)</t>
+          <t>📈 Trending (+213⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49943</v>
+        <v>49992</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4980</v>
+        <v>4988</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+21⭐)</t>
+          <t>📈 Trending (+49⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13971</v>
+        <v>13978</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1669</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+6⭐)</t>
+          <t>📈 Trending (+7⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10975</v>
+        <v>10981</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2600</v>
+        <v>2601</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>📈 Trending (+6⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5719</v>
+        <v>5720</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>271405</v>
+        <v>272314</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>40545</v>
+        <v>40663</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>151885</v>
+        <v>153541</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8145</v>
+        <v>8246</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>123353</v>
+        <v>123574</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11888</v>
+        <v>11911</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+245⭐)</t>
+          <t>📈 Trending (+221⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95644</v>
+        <v>95649</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9586</v>
+        <v>9588</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+5⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>89828</v>
+        <v>89919</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11864</v>
+        <v>11878</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+70⭐)</t>
+          <t>📈 Trending (+91⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>216595</v>
+        <v>216731</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21810</v>
+        <v>21820</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+136⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187639</v>
+        <v>187642</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45959</v>
+        <v>45957</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>182069</v>
+        <v>182131</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18085</v>
+        <v>18096</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+40⭐)</t>
+          <t>📈 Trending (+62⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>187981</v>
+        <v>188316</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10008</v>
+        <v>10020</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>🔥 Supercharge your AI agents with data from the web and beyond. A web data API to search, scrape, and access more sources.</t>
+          <t>Supercharge your AI agents with data from the web and beyond. Building the library for superintelligence. 🔥</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>82255</v>
+        <v>82315</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5223</v>
+        <v>5233</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+73⭐)</t>
+          <t>📈 Trending (+60⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-05]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>251001</v>
+        <v>251255</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>53828</v>
+        <v>53927</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157788</v>
+        <v>157853</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24899</v>
+        <v>24906</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+55⭐)</t>
+          <t>📈 Trending (+65⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155488</v>
+        <v>155504</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10175</v>
+        <v>10178</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+28⭐)</t>
+          <t>📈 Trending (+16⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>156041</v>
+        <v>156700</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25176</v>
+        <v>25284</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+213⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>49992</v>
+        <v>50038</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4988</v>
+        <v>4997</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+49⭐)</t>
+          <t>📈 Trending (+46⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13978</v>
+        <v>13979</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1669</v>
+        <v>1674</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+7⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10981</v>
+        <v>10984</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2601</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+6⭐)</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6239</v>
+        <v>6240</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>272314</v>
+        <v>273015</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>40663</v>
+        <v>40748</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>153541</v>
+        <v>154969</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8246</v>
+        <v>8329</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>123574</v>
+        <v>123812</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11911</v>
+        <v>11941</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+221⭐)</t>
+          <t>📈 Trending (+238⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95649</v>
+        <v>95656</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9588</v>
+        <v>9587</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+5⭐)</t>
+          <t>📈 Trending (+7⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>89919</v>
+        <v>90002</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11878</v>
+        <v>11895</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+91⭐)</t>
+          <t>📈 Trending (+83⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>216731</v>
+        <v>216883</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21820</v>
+        <v>21842</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+136⭐)</t>
+          <t>📈 Trending (+152⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187642</v>
+        <v>187660</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>45957</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>📈 Trending (+18⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>182131</v>
+        <v>182207</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18096</v>
+        <v>18102</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+62⭐)</t>
+          <t>📈 Trending (+76⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>188316</v>
+        <v>188631</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10020</v>
+        <v>10022</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>82315</v>
+        <v>82382</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5233</v>
+        <v>5243</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+60⭐)</t>
+          <t>📈 Trending (+67⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-06]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>251255</v>
+        <v>251474</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>53927</v>
+        <v>54014</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157853</v>
+        <v>157910</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24906</v>
+        <v>24915</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+65⭐)</t>
+          <t>📈 Trending (+57⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155504</v>
+        <v>155523</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10178</v>
+        <v>10185</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+16⭐)</t>
+          <t>📈 Trending (+19⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>156700</v>
+        <v>157333</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25284</v>
+        <v>25375</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50038</v>
+        <v>50072</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>4997</v>
+        <v>5001</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+46⭐)</t>
+          <t>📈 Trending (+34⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13979</v>
+        <v>13993</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+14⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10984</v>
+        <v>10983</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2601</v>
+        <v>2602</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6240</v>
+        <v>6239</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5720</v>
+        <v>5721</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>715</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>273015</v>
+        <v>273713</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>40748</v>
+        <v>40841</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>154969</v>
+        <v>156077</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8329</v>
+        <v>8389</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>123812</v>
+        <v>124079</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11941</v>
+        <v>11974</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+238⭐)</t>
+          <t>📈 Trending (+267⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95656</v>
+        <v>95658</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9587</v>
+        <v>9585</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+7⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>90002</v>
+        <v>90068</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11895</v>
+        <v>11910</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+83⭐)</t>
+          <t>📈 Trending (+66⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>216883</v>
+        <v>217095</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21842</v>
+        <v>21857</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+152⭐)</t>
+          <t>📈 Trending (+212⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187660</v>
+        <v>187663</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45957</v>
+        <v>45949</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+18⭐)</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>182207</v>
+        <v>182276</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18102</v>
+        <v>18109</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+76⭐)</t>
+          <t>📈 Trending (+69⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>188631</v>
+        <v>188951</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10022</v>
+        <v>10029</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>82382</v>
+        <v>82465</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5243</v>
+        <v>5249</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+67⭐)</t>
+          <t>📈 Trending (+83⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-07]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>251474</v>
+        <v>251725</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>54014</v>
+        <v>54126</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157910</v>
+        <v>157974</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24915</v>
+        <v>24927</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+57⭐)</t>
+          <t>📈 Trending (+64⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155523</v>
+        <v>155549</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10185</v>
+        <v>10188</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+19⭐)</t>
+          <t>📈 Trending (+26⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>157333</v>
+        <v>157874</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25375</v>
+        <v>25452</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50072</v>
+        <v>50104</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5001</v>
+        <v>5008</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+34⭐)</t>
+          <t>📈 Trending (+32⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13993</v>
+        <v>13994</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1675</v>
+        <v>1678</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+14⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10983</v>
+        <v>10985</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2602</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>3874</v>
+        <v>3873</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>466</v>
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>273713</v>
+        <v>274346</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>40841</v>
+        <v>40933</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>156077</v>
+        <v>156914</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8389</v>
+        <v>8424</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>124079</v>
+        <v>124436</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11974</v>
+        <v>12000</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+267⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95658</v>
+        <v>95665</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9585</v>
+        <v>9587</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+7⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>90068</v>
+        <v>90125</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11910</v>
+        <v>11926</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+66⭐)</t>
+          <t>📈 Trending (+57⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>217095</v>
+        <v>217294</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21857</v>
+        <v>21880</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+212⭐)</t>
+          <t>📈 Trending (+199⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187663</v>
+        <v>187677</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45949</v>
+        <v>45940</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>📈 Trending (+14⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>182276</v>
+        <v>182410</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18109</v>
+        <v>18123</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+69⭐)</t>
+          <t>📈 Trending (+134⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>188951</v>
+        <v>189237</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10029</v>
+        <v>10043</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>82465</v>
+        <v>82567</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5249</v>
+        <v>5251</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+83⭐)</t>
+          <t>📈 Trending (+102⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-08]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>251725</v>
+        <v>251981</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>54126</v>
+        <v>54262</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157974</v>
+        <v>158051</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24927</v>
+        <v>24939</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+64⭐)</t>
+          <t>📈 Trending (+77⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155549</v>
+        <v>155571</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10188</v>
+        <v>10193</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+26⭐)</t>
+          <t>📈 Trending (+22⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>157874</v>
+        <v>158304</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25452</v>
+        <v>25509</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50104</v>
+        <v>50137</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5008</v>
+        <v>5016</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+32⭐)</t>
+          <t>📈 Trending (+33⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>13994</v>
+        <v>14007</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1678</v>
+        <v>1681</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+13⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10985</v>
+        <v>10986</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2602</v>
+        <v>2603</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>274346</v>
+        <v>274994</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>40933</v>
+        <v>41025</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>156914</v>
+        <v>157694</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8424</v>
+        <v>8471</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>124436</v>
+        <v>124712</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12000</v>
+        <v>12020</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+276⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95665</v>
+        <v>95669</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9587</v>
+        <v>9588</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+7⭐)</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>90125</v>
+        <v>90217</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11926</v>
+        <v>11940</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+57⭐)</t>
+          <t>📈 Trending (+92⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>217294</v>
+        <v>217463</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21880</v>
+        <v>21891</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+199⭐)</t>
+          <t>📈 Trending (+169⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,10 +1384,10 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187677</v>
+        <v>187691</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45940</v>
+        <v>45938</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>182410</v>
+        <v>182512</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18123</v>
+        <v>18147</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+134⭐)</t>
+          <t>📈 Trending (+102⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>189237</v>
+        <v>189538</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10043</v>
+        <v>10046</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>82567</v>
+        <v>82645</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5251</v>
+        <v>5252</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+102⭐)</t>
+          <t>📈 Trending (+78⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-09]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>251981</v>
+        <v>252070</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>54262</v>
+        <v>54393</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158051</v>
+        <v>157939</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24939</v>
+        <v>24947</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+77⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155571</v>
+        <v>155407</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10193</v>
+        <v>10191</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+22⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>158304</v>
+        <v>158357</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25509</v>
+        <v>25548</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+53⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50137</v>
+        <v>50200</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5016</v>
+        <v>5020</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+33⭐)</t>
+          <t>📈 Trending (+63⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14007</v>
+        <v>14019</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1681</v>
+        <v>1682</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+13⭐)</t>
+          <t>📈 Trending (+12⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1000,7 +1000,7 @@
         <v>5721</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>3873</v>
+        <v>3871</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>466</v>
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>274994</v>
+        <v>275462</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>41025</v>
+        <v>41118</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>157694</v>
+        <v>158657</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8471</v>
+        <v>8531</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>124712</v>
+        <v>124778</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12020</v>
+        <v>12050</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+276⭐)</t>
+          <t>📈 Trending (+66⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95669</v>
+        <v>95670</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9588</v>
+        <v>9587</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+4⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>90217</v>
+        <v>90313</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11940</v>
+        <v>11952</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+92⭐)</t>
+          <t>📈 Trending (+96⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>217463</v>
+        <v>217478</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21891</v>
+        <v>21911</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+169⭐)</t>
+          <t>📈 Trending (+15⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187691</v>
+        <v>187489</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45938</v>
+        <v>45934</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+14⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>182512</v>
+        <v>182425</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18147</v>
+        <v>18168</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+102⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>189538</v>
+        <v>189653</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10046</v>
+        <v>10061</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>82645</v>
+        <v>82719</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5252</v>
+        <v>5251</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+78⭐)</t>
+          <t>📈 Trending (+74⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-10]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>252070</v>
+        <v>252307</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>54393</v>
+        <v>54508</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>157939</v>
+        <v>158033</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24947</v>
+        <v>24950</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+94⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155407</v>
+        <v>155448</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10191</v>
+        <v>10192</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+41⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>158357</v>
+        <v>158546</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25548</v>
+        <v>25584</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+53⭐)</t>
+          <t>📈 Trending (+189⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50200</v>
+        <v>50226</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5020</v>
+        <v>5026</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+63⭐)</t>
+          <t>📈 Trending (+26⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14019</v>
+        <v>14029</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1682</v>
+        <v>1683</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+12⭐)</t>
+          <t>📈 Trending (+10⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10986</v>
+        <v>10981</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2603</v>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6239</v>
+        <v>6240</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>275462</v>
+        <v>276034</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>41118</v>
+        <v>41183</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>158657</v>
+        <v>159713</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8531</v>
+        <v>8591</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>124778</v>
+        <v>125058</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12050</v>
+        <v>12074</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+66⭐)</t>
+          <t>📈 Trending (+280⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95670</v>
+        <v>95672</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9587</v>
+        <v>9590</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>90313</v>
+        <v>90425</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11952</v>
+        <v>11961</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+96⭐)</t>
+          <t>📈 Trending (+112⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>217478</v>
+        <v>217763</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21911</v>
+        <v>21950</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+15⭐)</t>
+          <t>📈 Trending (+285⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187489</v>
+        <v>187500</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45934</v>
+        <v>45927</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+11⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>182425</v>
+        <v>182551</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18168</v>
+        <v>18179</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+126⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>189653</v>
+        <v>189965</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10061</v>
+        <v>10076</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>82719</v>
+        <v>82799</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5251</v>
+        <v>5255</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+74⭐)</t>
+          <t>📈 Trending (+80⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-11]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>252307</v>
+        <v>252565</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>54508</v>
+        <v>54607</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158033</v>
+        <v>158104</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24950</v>
+        <v>24966</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+94⭐)</t>
+          <t>📈 Trending (+71⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155448</v>
+        <v>155482</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10192</v>
+        <v>10199</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+41⭐)</t>
+          <t>📈 Trending (+34⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>158546</v>
+        <v>158807</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25584</v>
+        <v>25638</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+189⭐)</t>
+          <t>📈 Trending (+261⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50226</v>
+        <v>50259</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5026</v>
+        <v>5032</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+26⭐)</t>
+          <t>📈 Trending (+33⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,10 +868,10 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14029</v>
+        <v>14039</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1683</v>
+        <v>1684</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10981</v>
+        <v>10980</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2603</v>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6240</v>
+        <v>6241</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1040,14 +1040,14 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>3871</v>
+        <v>3872</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>466</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>276034</v>
+        <v>276573</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>41183</v>
+        <v>41244</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>159713</v>
+        <v>160511</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8591</v>
+        <v>8631</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>125058</v>
+        <v>125328</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12074</v>
+        <v>12100</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+280⭐)</t>
+          <t>📈 Trending (+270⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95672</v>
+        <v>95676</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9590</v>
+        <v>9589</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>90425</v>
+        <v>90527</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11961</v>
+        <v>11985</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+112⭐)</t>
+          <t>📈 Trending (+102⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>217763</v>
+        <v>218334</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21950</v>
+        <v>21985</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+285⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187500</v>
+        <v>187518</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45927</v>
+        <v>45924</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+11⭐)</t>
+          <t>📈 Trending (+18⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>182551</v>
+        <v>182670</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18179</v>
+        <v>18195</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+126⭐)</t>
+          <t>📈 Trending (+119⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>189965</v>
+        <v>190239</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10076</v>
+        <v>10090</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1513,14 +1513,14 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>82799</v>
+        <v>82882</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5255</v>
+        <v>5258</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+80⭐)</t>
+          <t>📈 Trending (+83⭐)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-12]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>252565</v>
+        <v>252844</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>54607</v>
+        <v>54757</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158104</v>
+        <v>158179</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>24966</v>
+        <v>25006</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+71⭐)</t>
+          <t>📈 Trending (+75⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155482</v>
+        <v>155518</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10199</v>
+        <v>10230</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+34⭐)</t>
+          <t>📈 Trending (+36⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>158807</v>
+        <v>159167</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25638</v>
+        <v>25719</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+261⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50259</v>
+        <v>50294</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5032</v>
+        <v>5039</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+33⭐)</t>
+          <t>📈 Trending (+35⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14039</v>
+        <v>14054</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+10⭐)</t>
+          <t>📈 Trending (+15⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10980</v>
+        <v>10981</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2603</v>
+        <v>2600</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6241</v>
+        <v>6239</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1000,7 +1000,7 @@
         <v>5721</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>276573</v>
+        <v>277303</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>41244</v>
+        <v>41360</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>160511</v>
+        <v>161183</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8631</v>
+        <v>8697</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>125328</v>
+        <v>125588</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12100</v>
+        <v>12122</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+270⭐)</t>
+          <t>📈 Trending (+260⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95676</v>
+        <v>95680</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>9589</v>
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,10 +1255,10 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>90527</v>
+        <v>90629</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>11985</v>
+        <v>12002</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>218334</v>
+        <v>218942</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>21985</v>
+        <v>22055</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187518</v>
+        <v>187527</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45924</v>
+        <v>45948</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+18⭐)</t>
+          <t>📈 Trending (+9⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>182670</v>
+        <v>182794</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18195</v>
+        <v>18223</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+119⭐)</t>
+          <t>📈 Trending (+124⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>190239</v>
+        <v>190561</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10090</v>
+        <v>10123</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1546,6 +1546,59 @@
       <c r="K25" s="4" t="inlineStr">
         <is>
           <t>https://github.com/rtk-ai/rtk</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>🛠️ Developer Tools &amp; Powerful CLIs</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>morluto/rea</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>110669</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>24615</v>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>✨ Featured</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>TypeScript</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>Reverse engineer anything with agents, from app behavior down to native binaries.</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>Build Autonomous AI Agents &amp; Multi-Agent Workflows</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>agent-skills, ai-agents, binary-analysis, claude-code, cli</t>
+        </is>
+      </c>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/morluto/rea</t>
         </is>
       </c>
     </row>
@@ -1574,6 +1627,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-13]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>252844</v>
+        <v>253193</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>54757</v>
+        <v>54880</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158179</v>
+        <v>158300</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25006</v>
+        <v>25015</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+75⭐)</t>
+          <t>📈 Trending (+121⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155518</v>
+        <v>155575</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10230</v>
+        <v>10246</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+36⭐)</t>
+          <t>📈 Trending (+57⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>159167</v>
+        <v>159590</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25719</v>
+        <v>25790</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50294</v>
+        <v>50330</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5039</v>
+        <v>5043</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+35⭐)</t>
+          <t>📈 Trending (+36⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14054</v>
+        <v>14068</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+15⭐)</t>
+          <t>📈 Trending (+14⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10981</v>
+        <v>10982</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2600</v>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6239</v>
+        <v>6240</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5721</v>
+        <v>5720</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>715</v>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>277303</v>
+        <v>278017</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>41360</v>
+        <v>41441</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>161183</v>
+        <v>161983</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8697</v>
+        <v>8742</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>125588</v>
+        <v>125922</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12122</v>
+        <v>12153</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+260⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95680</v>
+        <v>95683</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9589</v>
+        <v>9590</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+4⭐)</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>90629</v>
+        <v>90763</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12002</v>
+        <v>12024</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+102⭐)</t>
+          <t>📈 Trending (+134⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>218942</v>
+        <v>219285</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22055</v>
+        <v>22074</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187527</v>
+        <v>187540</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45948</v>
+        <v>45941</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+9⭐)</t>
+          <t>📈 Trending (+13⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1427,14 +1427,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>182794</v>
+        <v>182940</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>18223</v>
+        <v>18246</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+124⭐)</t>
+          <t>📈 Trending (+146⭐)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>190561</v>
+        <v>190908</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10123</v>
+        <v>10134</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,14 +1566,14 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>110669</v>
+        <v>167321</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>24615</v>
+        <v>39701</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>🔥 Supernova (+1000⭐)</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-14]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>253193</v>
+        <v>253517</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>54880</v>
+        <v>54987</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158300</v>
+        <v>158391</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25015</v>
+        <v>25046</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+121⭐)</t>
+          <t>📈 Trending (+91⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,10 +653,10 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155575</v>
+        <v>155632</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10246</v>
+        <v>10248</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>159590</v>
+        <v>159911</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25790</v>
+        <v>25861</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50330</v>
+        <v>50355</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5043</v>
+        <v>5055</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+36⭐)</t>
+          <t>📈 Trending (+25⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14068</v>
+        <v>14084</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+14⭐)</t>
+          <t>📈 Trending (+16⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10982</v>
+        <v>10983</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2600</v>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>278017</v>
+        <v>278646</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>41441</v>
+        <v>41501</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>161983</v>
+        <v>162816</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8742</v>
+        <v>8798</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>125922</v>
+        <v>126221</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12153</v>
+        <v>12181</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+299⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95683</v>
+        <v>95688</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9590</v>
+        <v>9591</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>📈 Trending (+5⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>90763</v>
+        <v>90836</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12024</v>
+        <v>12039</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+134⭐)</t>
+          <t>📈 Trending (+73⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>219285</v>
+        <v>219519</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22074</v>
+        <v>22094</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+234⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187540</v>
+        <v>187564</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>45941</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+13⭐)</t>
+          <t>📈 Trending (+24⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>190908</v>
+        <v>191247</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10134</v>
+        <v>10145</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,14 +1566,14 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>167321</v>
+        <v>210700</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>39701</v>
+        <v>51680</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>🔥 Supernova (+1000⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-15]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>253517</v>
+        <v>253819</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>54987</v>
+        <v>55068</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158391</v>
+        <v>158497</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25046</v>
+        <v>25041</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+91⭐)</t>
+          <t>📈 Trending (+106⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155632</v>
+        <v>155678</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10248</v>
+        <v>10224</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+57⭐)</t>
+          <t>📈 Trending (+46⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>159911</v>
+        <v>160114</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25861</v>
+        <v>25879</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+203⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50355</v>
+        <v>50394</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5055</v>
+        <v>5056</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+25⭐)</t>
+          <t>📈 Trending (+39⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14084</v>
+        <v>14098</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1687</v>
+        <v>1696</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+16⭐)</t>
+          <t>📈 Trending (+14⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10983</v>
+        <v>10987</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2600</v>
+        <v>2599</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6240</v>
+        <v>6241</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>278646</v>
+        <v>279513</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>41501</v>
+        <v>41597</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>162816</v>
+        <v>163662</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8798</v>
+        <v>8821</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>126221</v>
+        <v>126570</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12181</v>
+        <v>12213</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+299⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95688</v>
+        <v>95697</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9591</v>
+        <v>9590</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+5⭐)</t>
+          <t>📈 Trending (+9⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>90836</v>
+        <v>90921</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12039</v>
+        <v>12051</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+73⭐)</t>
+          <t>📈 Trending (+85⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>219519</v>
+        <v>219836</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22094</v>
+        <v>22105</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+234⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187564</v>
+        <v>187579</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45941</v>
+        <v>45922</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+24⭐)</t>
+          <t>📈 Trending (+15⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>191247</v>
+        <v>191602</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10145</v>
+        <v>10130</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>210700</v>
+        <v>244318</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>51680</v>
+        <v>61035</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-16]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>253819</v>
+        <v>254136</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>55068</v>
+        <v>55188</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158497</v>
+        <v>158593</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25041</v>
+        <v>25055</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+106⭐)</t>
+          <t>📈 Trending (+96⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155678</v>
+        <v>155721</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10224</v>
+        <v>10236</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+46⭐)</t>
+          <t>📈 Trending (+43⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>160114</v>
+        <v>160365</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25879</v>
+        <v>25927</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+203⭐)</t>
+          <t>📈 Trending (+251⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50394</v>
+        <v>50418</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5056</v>
+        <v>5060</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+39⭐)</t>
+          <t>📈 Trending (+24⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14098</v>
+        <v>14117</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1696</v>
+        <v>1703</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+14⭐)</t>
+          <t>📈 Trending (+19⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10987</v>
+        <v>10990</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2599</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+4⭐)</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5720</v>
+        <v>5721</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>715</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>279513</v>
+        <v>280443</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>41597</v>
+        <v>41710</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>163662</v>
+        <v>164464</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8821</v>
+        <v>8866</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>126570</v>
+        <v>126928</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12213</v>
+        <v>12242</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95697</v>
+        <v>95701</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9590</v>
+        <v>9593</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+9⭐)</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>90921</v>
+        <v>91004</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12051</v>
+        <v>12064</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+85⭐)</t>
+          <t>📈 Trending (+83⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>219836</v>
+        <v>220110</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22105</v>
+        <v>22126</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+274⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187579</v>
+        <v>187599</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45922</v>
+        <v>45921</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+15⭐)</t>
+          <t>📈 Trending (+20⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>191602</v>
+        <v>191917</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10130</v>
+        <v>10146</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>244318</v>
+        <v>271836</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>61035</v>
+        <v>68316</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-17]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>254136</v>
+        <v>254443</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>55188</v>
+        <v>55277</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158593</v>
+        <v>158671</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25055</v>
+        <v>25078</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+96⭐)</t>
+          <t>📈 Trending (+78⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155721</v>
+        <v>155759</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10236</v>
+        <v>10238</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+43⭐)</t>
+          <t>📈 Trending (+38⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>160365</v>
+        <v>160608</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25927</v>
+        <v>25968</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+251⭐)</t>
+          <t>📈 Trending (+243⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50418</v>
+        <v>50445</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5060</v>
+        <v>5061</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+24⭐)</t>
+          <t>📈 Trending (+27⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14117</v>
+        <v>14135</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1703</v>
+        <v>1722</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+19⭐)</t>
+          <t>📈 Trending (+18⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10990</v>
+        <v>10995</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2599</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>📈 Trending (+5⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6241</v>
+        <v>6242</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5721</v>
+        <v>5723</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>715</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>280443</v>
+        <v>281550</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>41710</v>
+        <v>41861</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>164464</v>
+        <v>165240</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8866</v>
+        <v>8924</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>126928</v>
+        <v>127267</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12242</v>
+        <v>12280</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95701</v>
+        <v>95711</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9593</v>
+        <v>9595</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+4⭐)</t>
+          <t>📈 Trending (+10⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91004</v>
+        <v>91078</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12064</v>
+        <v>12078</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+83⭐)</t>
+          <t>📈 Trending (+74⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>220110</v>
+        <v>220375</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22126</v>
+        <v>22147</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+274⭐)</t>
+          <t>📈 Trending (+265⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187599</v>
+        <v>187614</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45921</v>
+        <v>45918</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+20⭐)</t>
+          <t>📈 Trending (+15⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>191917</v>
+        <v>192222</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10146</v>
+        <v>10154</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>271836</v>
+        <v>291750</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>68316</v>
+        <v>73456</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-18]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>254443</v>
+        <v>254702</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>55277</v>
+        <v>55367</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158671</v>
+        <v>158730</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25078</v>
+        <v>25087</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+78⭐)</t>
+          <t>📈 Trending (+59⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155759</v>
+        <v>155782</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10238</v>
+        <v>10242</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+38⭐)</t>
+          <t>📈 Trending (+23⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>160608</v>
+        <v>160916</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>25968</v>
+        <v>26038</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+243⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50445</v>
+        <v>50458</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5061</v>
+        <v>5063</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+27⭐)</t>
+          <t>📈 Trending (+13⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,10 +868,10 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14135</v>
+        <v>14153</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1722</v>
+        <v>1778</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10995</v>
+        <v>10996</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2599</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+5⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6242</v>
+        <v>6241</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>281550</v>
+        <v>282546</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>41861</v>
+        <v>41988</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>165240</v>
+        <v>166269</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8924</v>
+        <v>8994</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>127267</v>
+        <v>127813</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12280</v>
+        <v>12317</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95711</v>
+        <v>95714</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>9595</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+10⭐)</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91078</v>
+        <v>91147</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12078</v>
+        <v>12092</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+74⭐)</t>
+          <t>📈 Trending (+69⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>220375</v>
+        <v>220667</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22147</v>
+        <v>22168</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+265⭐)</t>
+          <t>📈 Trending (+292⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187614</v>
+        <v>187630</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45918</v>
+        <v>45909</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+15⭐)</t>
+          <t>📈 Trending (+16⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>192222</v>
+        <v>192513</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10154</v>
+        <v>10168</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>291750</v>
+        <v>308295</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>73456</v>
+        <v>78014</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-19]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>254702</v>
+        <v>254965</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>55367</v>
+        <v>55473</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158730</v>
+        <v>158822</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25087</v>
+        <v>25100</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+59⭐)</t>
+          <t>📈 Trending (+92⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155782</v>
+        <v>155811</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10242</v>
+        <v>10251</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+23⭐)</t>
+          <t>📈 Trending (+29⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>160916</v>
+        <v>161222</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26038</v>
+        <v>26088</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50458</v>
+        <v>50479</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5063</v>
+        <v>5065</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+13⭐)</t>
+          <t>📈 Trending (+21⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14153</v>
+        <v>14172</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1778</v>
+        <v>1819</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+18⭐)</t>
+          <t>📈 Trending (+19⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10996</v>
+        <v>10994</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2599</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6241</v>
+        <v>6242</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5723</v>
+        <v>5722</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>715</v>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>3872</v>
+        <v>3871</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>466</v>
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>282546</v>
+        <v>283326</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>41988</v>
+        <v>42090</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>166269</v>
+        <v>167102</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8994</v>
+        <v>9071</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>127813</v>
+        <v>128453</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12317</v>
+        <v>12382</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95714</v>
+        <v>95720</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9595</v>
+        <v>9597</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>📈 Trending (+6⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91147</v>
+        <v>91221</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12092</v>
+        <v>12108</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+69⭐)</t>
+          <t>📈 Trending (+74⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>220667</v>
+        <v>220979</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22168</v>
+        <v>22197</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+292⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187630</v>
+        <v>187644</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45909</v>
+        <v>45914</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+16⭐)</t>
+          <t>📈 Trending (+14⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>192513</v>
+        <v>192807</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10168</v>
+        <v>10183</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>308295</v>
+        <v>323228</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>78014</v>
+        <v>81899</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-20]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>254965</v>
+        <v>255298</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>55473</v>
+        <v>55581</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158822</v>
+        <v>158944</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25100</v>
+        <v>25121</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+92⭐)</t>
+          <t>📈 Trending (+122⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155811</v>
+        <v>155852</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10251</v>
+        <v>10260</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+29⭐)</t>
+          <t>📈 Trending (+41⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>161222</v>
+        <v>161805</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26088</v>
+        <v>26182</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50479</v>
+        <v>50509</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5065</v>
+        <v>5068</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+21⭐)</t>
+          <t>📈 Trending (+30⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14172</v>
+        <v>14192</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1819</v>
+        <v>1851</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+19⭐)</t>
+          <t>📈 Trending (+20⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10994</v>
+        <v>10992</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2599</v>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>3871</v>
+        <v>3870</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>466</v>
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>283326</v>
+        <v>284179</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>42090</v>
+        <v>42212</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>167102</v>
+        <v>168167</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9071</v>
+        <v>9144</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>128453</v>
+        <v>129223</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12382</v>
+        <v>12461</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95720</v>
+        <v>95727</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9597</v>
+        <v>9600</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+6⭐)</t>
+          <t>📈 Trending (+7⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91221</v>
+        <v>91310</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12108</v>
+        <v>12121</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+74⭐)</t>
+          <t>📈 Trending (+89⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>220979</v>
+        <v>221247</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22197</v>
+        <v>22226</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+268⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187644</v>
+        <v>187661</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45914</v>
+        <v>45917</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+14⭐)</t>
+          <t>📈 Trending (+17⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>192807</v>
+        <v>193124</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10183</v>
+        <v>10196</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>323228</v>
+        <v>337642</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>81899</v>
+        <v>85254</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-21]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>255298</v>
+        <v>255610</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>55581</v>
+        <v>55700</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>158944</v>
+        <v>159073</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25121</v>
+        <v>25140</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+122⭐)</t>
+          <t>📈 Trending (+129⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155852</v>
+        <v>155872</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10260</v>
+        <v>10236</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+41⭐)</t>
+          <t>📈 Trending (+20⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>161805</v>
+        <v>162405</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26182</v>
+        <v>26231</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50509</v>
+        <v>50533</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5068</v>
+        <v>5077</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+30⭐)</t>
+          <t>📈 Trending (+24⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14192</v>
+        <v>14214</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1851</v>
+        <v>1726</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+20⭐)</t>
+          <t>📈 Trending (+22⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10992</v>
+        <v>10993</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2599</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1000,7 +1000,7 @@
         <v>5722</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>284179</v>
+        <v>284942</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>42212</v>
+        <v>42280</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>168167</v>
+        <v>169828</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9144</v>
+        <v>9234</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>129223</v>
+        <v>130339</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12461</v>
+        <v>12546</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>🔥 Supernova (+1000⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95727</v>
+        <v>95726</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9600</v>
+        <v>9579</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+7⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91310</v>
+        <v>91418</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12121</v>
+        <v>12131</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+89⭐)</t>
+          <t>📈 Trending (+108⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,14 +1341,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>221247</v>
+        <v>221553</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22226</v>
+        <v>22245</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+268⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187661</v>
+        <v>187679</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45917</v>
+        <v>45915</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+17⭐)</t>
+          <t>📈 Trending (+18⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>193124</v>
+        <v>193509</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10196</v>
+        <v>10212</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>337642</v>
+        <v>348705</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>85254</v>
+        <v>87716</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-22]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>255610</v>
+        <v>255981</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>55700</v>
+        <v>55841</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>159073</v>
+        <v>159166</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25140</v>
+        <v>25155</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+129⭐)</t>
+          <t>📈 Trending (+93⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155872</v>
+        <v>155900</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10236</v>
+        <v>10230</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+20⭐)</t>
+          <t>📈 Trending (+28⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>162405</v>
+        <v>162961</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26231</v>
+        <v>26293</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50533</v>
+        <v>50559</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5077</v>
+        <v>5078</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+24⭐)</t>
+          <t>📈 Trending (+26⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,10 +868,10 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14214</v>
+        <v>14236</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1726</v>
+        <v>1709</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,10 +911,10 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10993</v>
+        <v>10994</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2599</v>
+        <v>2600</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6242</v>
+        <v>6243</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>284942</v>
+        <v>285769</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>42280</v>
+        <v>42389</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>169828</v>
+        <v>171764</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9234</v>
+        <v>9346</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>130339</v>
+        <v>131727</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12546</v>
+        <v>12645</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95726</v>
+        <v>95730</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9579</v>
+        <v>9571</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91418</v>
+        <v>91502</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12131</v>
+        <v>12145</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+108⭐)</t>
+          <t>📈 Trending (+84⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>221553</v>
+        <v>221979</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22245</v>
+        <v>22269</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187679</v>
+        <v>187704</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45915</v>
+        <v>45908</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+18⭐)</t>
+          <t>📈 Trending (+25⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>193509</v>
+        <v>193960</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10212</v>
+        <v>10232</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>348705</v>
+        <v>358339</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>87716</v>
+        <v>89933</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-23]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>255981</v>
+        <v>256271</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>55841</v>
+        <v>55977</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>159166</v>
+        <v>159295</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25155</v>
+        <v>25165</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+93⭐)</t>
+          <t>📈 Trending (+129⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155900</v>
+        <v>155935</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10230</v>
+        <v>10240</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+28⭐)</t>
+          <t>📈 Trending (+35⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>162961</v>
+        <v>163294</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26293</v>
+        <v>26351</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50559</v>
+        <v>50589</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5078</v>
+        <v>5086</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+26⭐)</t>
+          <t>📈 Trending (+30⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14236</v>
+        <v>14329</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1709</v>
+        <v>1726</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+22⭐)</t>
+          <t>📈 Trending (+93⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5722</v>
+        <v>5723</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>285769</v>
+        <v>286577</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>42389</v>
+        <v>42511</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>171764</v>
+        <v>173609</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9346</v>
+        <v>9447</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>131727</v>
+        <v>133039</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12645</v>
+        <v>12728</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95730</v>
+        <v>95736</v>
       </c>
       <c r="E18" s="5" t="n">
         <v>9571</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+4⭐)</t>
+          <t>📈 Trending (+6⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91502</v>
+        <v>91597</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12145</v>
+        <v>12160</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+84⭐)</t>
+          <t>📈 Trending (+95⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>221979</v>
+        <v>222552</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22269</v>
+        <v>22316</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187704</v>
+        <v>187717</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45908</v>
+        <v>45905</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+25⭐)</t>
+          <t>📈 Trending (+13⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>193960</v>
+        <v>194331</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10232</v>
+        <v>10258</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>358339</v>
+        <v>366730</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>89933</v>
+        <v>91894</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-24]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>256271</v>
+        <v>256544</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>55977</v>
+        <v>56082</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>159295</v>
+        <v>159381</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25165</v>
+        <v>25177</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+129⭐)</t>
+          <t>📈 Trending (+86⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155935</v>
+        <v>155969</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10240</v>
+        <v>10242</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+35⭐)</t>
+          <t>📈 Trending (+34⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>163294</v>
+        <v>163526</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26351</v>
+        <v>26391</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+232⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50589</v>
+        <v>50636</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5086</v>
+        <v>5096</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+30⭐)</t>
+          <t>📈 Trending (+47⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14329</v>
+        <v>14344</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1726</v>
+        <v>1728</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+93⭐)</t>
+          <t>📈 Trending (+15⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10994</v>
+        <v>10998</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2600</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>286577</v>
+        <v>287379</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>42511</v>
+        <v>42615</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>173609</v>
+        <v>174836</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9447</v>
+        <v>9522</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,14 +1169,14 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>133039</v>
+        <v>133926</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12728</v>
+        <v>12794</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>🔥 Supernova (+1000⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95736</v>
+        <v>95740</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9571</v>
+        <v>9570</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+6⭐)</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91597</v>
+        <v>91681</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12160</v>
+        <v>12165</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+95⭐)</t>
+          <t>📈 Trending (+84⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>222552</v>
+        <v>222939</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22316</v>
+        <v>22346</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187717</v>
+        <v>187720</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45905</v>
+        <v>45898</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+13⭐)</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>194331</v>
+        <v>194704</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10258</v>
+        <v>10273</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>366730</v>
+        <v>373487</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>91894</v>
+        <v>93418</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-25]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>256544</v>
+        <v>256829</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>56082</v>
+        <v>56182</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>159381</v>
+        <v>159441</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25177</v>
+        <v>25195</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+86⭐)</t>
+          <t>📈 Trending (+60⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155969</v>
+        <v>155991</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10242</v>
+        <v>10239</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+34⭐)</t>
+          <t>📈 Trending (+22⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>163526</v>
+        <v>163728</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26391</v>
+        <v>26431</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+232⭐)</t>
+          <t>📈 Trending (+202⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50636</v>
+        <v>50684</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5096</v>
+        <v>5103</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+47⭐)</t>
+          <t>📈 Trending (+48⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14344</v>
+        <v>14365</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1728</v>
+        <v>1730</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+15⭐)</t>
+          <t>📈 Trending (+21⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10998</v>
+        <v>11001</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2600</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+4⭐)</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6243</v>
+        <v>6245</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,14 +997,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5723</v>
+        <v>5724</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>718</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>287379</v>
+        <v>288125</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>42615</v>
+        <v>42716</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>174836</v>
+        <v>175555</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9522</v>
+        <v>9570</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>133926</v>
+        <v>134496</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12794</v>
+        <v>12838</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95740</v>
+        <v>95741</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9570</v>
+        <v>9571</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+4⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91681</v>
+        <v>91758</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12165</v>
+        <v>12175</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+84⭐)</t>
+          <t>📈 Trending (+77⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>222939</v>
+        <v>223412</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22346</v>
+        <v>22381</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187720</v>
+        <v>187731</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45898</v>
+        <v>45895</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>📈 Trending (+11⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>194704</v>
+        <v>195032</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10273</v>
+        <v>10292</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>373487</v>
+        <v>379004</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>93418</v>
+        <v>94705</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-26]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>256829</v>
+        <v>257076</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>56182</v>
+        <v>56314</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>159441</v>
+        <v>159534</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25195</v>
+        <v>25213</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+60⭐)</t>
+          <t>📈 Trending (+93⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>155991</v>
+        <v>156021</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10239</v>
+        <v>10245</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+22⭐)</t>
+          <t>📈 Trending (+30⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>163728</v>
+        <v>164017</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26431</v>
+        <v>26474</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+202⭐)</t>
+          <t>📈 Trending (+289⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50684</v>
+        <v>50714</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5103</v>
+        <v>5106</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+48⭐)</t>
+          <t>📈 Trending (+30⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14365</v>
+        <v>14388</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1730</v>
+        <v>1732</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+21⭐)</t>
+          <t>📈 Trending (+23⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>11001</v>
+        <v>11003</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2600</v>
+        <v>2598</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,14 +954,14 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6245</v>
+        <v>6246</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1043,7 +1043,7 @@
         <v>3870</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>288125</v>
+        <v>288899</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>42716</v>
+        <v>42831</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>175555</v>
+        <v>176227</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9570</v>
+        <v>9626</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>134496</v>
+        <v>135309</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12838</v>
+        <v>12910</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,10 +1212,10 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95741</v>
+        <v>95742</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9571</v>
+        <v>9576</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91758</v>
+        <v>91838</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12175</v>
+        <v>12195</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+77⭐)</t>
+          <t>📈 Trending (+80⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>223412</v>
+        <v>223880</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22381</v>
+        <v>22415</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187731</v>
+        <v>187747</v>
       </c>
       <c r="E22" s="5" t="n">
         <v>45895</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+11⭐)</t>
+          <t>📈 Trending (+16⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>195032</v>
+        <v>195347</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10292</v>
+        <v>10305</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>379004</v>
+        <v>385021</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>94705</v>
+        <v>96402</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-27]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>257076</v>
+        <v>257445</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>56314</v>
+        <v>56415</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>159534</v>
+        <v>159641</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25213</v>
+        <v>25228</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+93⭐)</t>
+          <t>📈 Trending (+107⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>156021</v>
+        <v>156044</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10245</v>
+        <v>10250</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+30⭐)</t>
+          <t>📈 Trending (+23⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>164017</v>
+        <v>164289</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26474</v>
+        <v>26505</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+289⭐)</t>
+          <t>📈 Trending (+272⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50714</v>
+        <v>50769</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5106</v>
+        <v>5115</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+30⭐)</t>
+          <t>📈 Trending (+55⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14388</v>
+        <v>14405</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>1732</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+23⭐)</t>
+          <t>📈 Trending (+17⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,10 +911,10 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>11003</v>
+        <v>11005</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2598</v>
+        <v>2597</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1040,14 +1040,14 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>3870</v>
+        <v>3871</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>465</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>288899</v>
+        <v>289926</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>42831</v>
+        <v>42965</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>176227</v>
+        <v>177248</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9626</v>
+        <v>9693</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>135309</v>
+        <v>136222</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>12910</v>
+        <v>13004</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95742</v>
+        <v>95745</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9576</v>
+        <v>9581</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>📈 Trending (+3⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91838</v>
+        <v>91942</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12195</v>
+        <v>12213</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+80⭐)</t>
+          <t>📈 Trending (+104⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>223880</v>
+        <v>224730</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22415</v>
+        <v>22479</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187747</v>
+        <v>187781</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45895</v>
+        <v>45903</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+16⭐)</t>
+          <t>📈 Trending (+34⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>195347</v>
+        <v>195721</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10305</v>
+        <v>10330</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>385021</v>
+        <v>392186</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>96402</v>
+        <v>98276</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-28]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>257445</v>
+        <v>257779</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>56415</v>
+        <v>56536</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>159641</v>
+        <v>159744</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25228</v>
+        <v>25243</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+107⭐)</t>
+          <t>📈 Trending (+103⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>156044</v>
+        <v>156074</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10250</v>
+        <v>10253</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+23⭐)</t>
+          <t>📈 Trending (+30⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>164289</v>
+        <v>164566</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26505</v>
+        <v>26538</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+272⭐)</t>
+          <t>📈 Trending (+277⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50769</v>
+        <v>50815</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5115</v>
+        <v>5120</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+55⭐)</t>
+          <t>📈 Trending (+46⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14405</v>
+        <v>14425</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1732</v>
+        <v>1737</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+17⭐)</t>
+          <t>📈 Trending (+20⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>11005</v>
+        <v>11006</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2597</v>
+        <v>2595</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+1⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6246</v>
+        <v>6245</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,10 +997,10 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5724</v>
+        <v>5723</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1040,14 +1040,14 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>3871</v>
+        <v>3870</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>465</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>289926</v>
+        <v>290972</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>42965</v>
+        <v>43085</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>177248</v>
+        <v>178273</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9693</v>
+        <v>9760</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>136222</v>
+        <v>137061</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>13004</v>
+        <v>13078</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95745</v>
+        <v>95755</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9581</v>
+        <v>9584</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+3⭐)</t>
+          <t>📈 Trending (+10⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>91942</v>
+        <v>92040</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12213</v>
+        <v>12228</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+104⭐)</t>
+          <t>📈 Trending (+98⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>224730</v>
+        <v>225542</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22479</v>
+        <v>22530</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187781</v>
+        <v>187792</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45903</v>
+        <v>45901</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+34⭐)</t>
+          <t>📈 Trending (+11⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>195721</v>
+        <v>196110</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10330</v>
+        <v>10360</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>392186</v>
+        <v>397833</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>98276</v>
+        <v>99769</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-29]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>257779</v>
+        <v>258103</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>56536</v>
+        <v>56650</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>159744</v>
+        <v>159854</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25243</v>
+        <v>25254</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+103⭐)</t>
+          <t>📈 Trending (+110⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>156074</v>
+        <v>156121</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10253</v>
+        <v>10260</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+30⭐)</t>
+          <t>📈 Trending (+47⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>164566</v>
+        <v>164914</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26538</v>
+        <v>26622</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+277⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50815</v>
+        <v>50857</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5120</v>
+        <v>5128</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+46⭐)</t>
+          <t>📈 Trending (+42⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,10 +868,10 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14425</v>
+        <v>14445</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1737</v>
+        <v>1738</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+1⭐)</t>
+          <t>✨ Featured</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5723</v>
+        <v>5722</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>717</v>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>3870</v>
+        <v>3869</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>465</v>
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>290972</v>
+        <v>291848</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>43085</v>
+        <v>43203</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>178273</v>
+        <v>179294</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9760</v>
+        <v>9827</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>137061</v>
+        <v>137950</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>13078</v>
+        <v>13151</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95755</v>
+        <v>95764</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9584</v>
+        <v>9583</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+10⭐)</t>
+          <t>📈 Trending (+9⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>92040</v>
+        <v>92132</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12228</v>
+        <v>12250</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+98⭐)</t>
+          <t>📈 Trending (+92⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>225542</v>
+        <v>226022</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22530</v>
+        <v>22579</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187792</v>
+        <v>187807</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45901</v>
+        <v>45895</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+11⭐)</t>
+          <t>📈 Trending (+15⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>196110</v>
+        <v>196457</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10360</v>
+        <v>10371</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>397833</v>
+        <v>403221</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>99769</v>
+        <v>101086</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-30]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>258103</v>
+        <v>258552</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>56650</v>
+        <v>56779</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>159854</v>
+        <v>159944</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25254</v>
+        <v>25268</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+110⭐)</t>
+          <t>📈 Trending (+90⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>156121</v>
+        <v>156147</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10260</v>
+        <v>10269</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+47⭐)</t>
+          <t>📈 Trending (+26⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>164914</v>
+        <v>165198</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26622</v>
+        <v>26685</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>⚡ Breakout (+300⭐)</t>
+          <t>📈 Trending (+284⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50857</v>
+        <v>50905</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5128</v>
+        <v>5131</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+42⭐)</t>
+          <t>📈 Trending (+48⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14445</v>
+        <v>14463</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1738</v>
+        <v>1742</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+20⭐)</t>
+          <t>📈 Trending (+18⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5722</v>
+        <v>5721</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>717</v>
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1040,10 +1040,10 @@
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>3869</v>
+        <v>3867</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>291848</v>
+        <v>292780</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>43203</v>
+        <v>43330</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>179294</v>
+        <v>180284</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9827</v>
+        <v>9889</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>137950</v>
+        <v>138787</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>13151</v>
+        <v>13234</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95764</v>
+        <v>95766</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9583</v>
+        <v>9590</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+9⭐)</t>
+          <t>📈 Trending (+2⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,14 +1255,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>92132</v>
+        <v>92215</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12250</v>
+        <v>12265</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+92⭐)</t>
+          <t>📈 Trending (+83⭐)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>226022</v>
+        <v>226496</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22579</v>
+        <v>22615</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187807</v>
+        <v>187820</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45895</v>
+        <v>45899</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+15⭐)</t>
+          <t>📈 Trending (+13⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>196457</v>
+        <v>196785</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10371</v>
+        <v>10387</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>403221</v>
+        <v>408369</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>101086</v>
+        <v>102264</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Auto Update: GitHub Daily Radar [2026-10-31]
</commit_message>
<xml_diff>
--- a/reports/github_radar_archive.xlsx
+++ b/reports/github_radar_archive.xlsx
@@ -553,7 +553,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>258552</v>
+        <v>258909</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>56779</v>
+        <v>56914</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -610,14 +610,14 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>159944</v>
+        <v>160037</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>25268</v>
+        <v>25291</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+90⭐)</t>
+          <t>📈 Trending (+93⭐)</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -653,14 +653,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>156147</v>
+        <v>156175</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10269</v>
+        <v>10284</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+26⭐)</t>
+          <t>📈 Trending (+28⭐)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -696,14 +696,14 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>165198</v>
+        <v>165521</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>26685</v>
+        <v>26787</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+284⭐)</t>
+          <t>⚡ Breakout (+300⭐)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -811,7 +811,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -825,14 +825,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>50905</v>
+        <v>50940</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5131</v>
+        <v>5134</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>📈 Trending (+48⭐)</t>
+          <t>📈 Trending (+35⭐)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -868,14 +868,14 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>14463</v>
+        <v>14484</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1742</v>
+        <v>1745</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+18⭐)</t>
+          <t>📈 Trending (+21⭐)</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -911,14 +911,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>11006</v>
+        <v>11010</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2595</v>
+        <v>2593</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>✨ Featured</t>
+          <t>📈 Trending (+4⭐)</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -940,7 +940,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>6245</v>
+        <v>6244</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>302</v>
@@ -983,7 +983,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1069,7 +1069,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1083,10 +1083,10 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>292780</v>
+        <v>293449</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>43330</v>
+        <v>43425</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1126,10 +1126,10 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>180284</v>
+        <v>181019</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>9889</v>
+        <v>9950</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,10 +1169,10 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>138787</v>
+        <v>139529</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>13234</v>
+        <v>13314</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -1212,14 +1212,14 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>95766</v>
+        <v>95772</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9590</v>
+        <v>9596</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+2⭐)</t>
+          <t>📈 Trending (+6⭐)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1241,7 +1241,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1255,10 +1255,10 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>92215</v>
+        <v>92298</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>12265</v>
+        <v>12286</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1341,10 +1341,10 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>226496</v>
+        <v>226909</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>22615</v>
+        <v>22656</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -1384,14 +1384,14 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>187820</v>
+        <v>187840</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>45899</v>
+        <v>45909</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>📈 Trending (+13⭐)</t>
+          <t>📈 Trending (+20⭐)</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1456,7 +1456,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>196785</v>
+        <v>197143</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>10387</v>
+        <v>10413</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -1566,10 +1566,10 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>408369</v>
+        <v>412620</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>102264</v>
+        <v>103219</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>

</xml_diff>